<commit_message>
Add Codex10k opportunity tracker
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc4f361d364c54d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R3bf9715398124514"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R29274ae370d940d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rc389b981105b4e7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R29c6dd2279624948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4331feac32f443dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R24c822c27ce34002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R45518841e17d4c35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTA(Prospects!A2:A200)</x:f>
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -350,6 +350,9 @@
       <x:c r="N1" t="str">
         <x:v>Evidence URI</x:v>
       </x:c>
+      <x:c r="O1" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -387,11 +390,14 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Initialized</x:v>
-      </x:c>
-      <x:c r="M2" t="str"/>
+        <x:v>initialized</x:v>
+      </x:c>
+      <x:c r="M2"/>
       <x:c r="N2" t="str">
         <x:v>docs/research.md</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>No verified revenue yet</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -408,31 +414,49 @@
         <x:v>Lead ID</x:v>
       </x:c>
       <x:c r="B1" t="str">
+        <x:v>Created</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Label Namespace</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
         <x:v>Company</x:v>
       </x:c>
-      <x:c r="C1" t="str">
+      <x:c r="E1" t="str">
+        <x:v>Contact</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
         <x:v>Channel</x:v>
       </x:c>
-      <x:c r="D1" t="str">
+      <x:c r="G1" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
         <x:v>Segment</x:v>
       </x:c>
-      <x:c r="E1" t="str">
+      <x:c r="I1" t="str">
         <x:v>Problem Hypothesis</x:v>
       </x:c>
-      <x:c r="F1" t="str">
+      <x:c r="J1" t="str">
         <x:v>Offer</x:v>
       </x:c>
-      <x:c r="G1" t="str">
+      <x:c r="K1" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H1" t="str">
+      <x:c r="L1" t="str">
+        <x:v>Last Touch</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
         <x:v>Next Action</x:v>
       </x:c>
-      <x:c r="I1" t="str">
+      <x:c r="N1" t="str">
         <x:v>Follow-up Date</x:v>
       </x:c>
-      <x:c r="J1" t="str">
+      <x:c r="O1" t="str">
         <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -440,29 +464,233 @@
         <x:v>C10K-000</x:v>
       </x:c>
       <x:c r="B2" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
         <x:v>Internal</x:v>
       </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Workspace</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2" t="str">
         <x:v>Run setup</x:v>
       </x:c>
-      <x:c r="E2" t="str">
-        <x:v>Independent Codex10k pipeline initialized</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
+      <x:c r="J2" t="str">
         <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
       </x:c>
-      <x:c r="G2" t="str">
-        <x:v>Initialized</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
+      <x:c r="K2" t="str">
+        <x:v>initialized</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
         <x:v>Begin fresh lead sourcing</x:v>
       </x:c>
-      <x:c r="I2" t="str"/>
-      <x:c r="J2" t="str">
+      <x:c r="N2"/>
+      <x:c r="O2" t="str">
         <x:v>docs/research.md</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>Do not mix with prior Revenue Run labels</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>C10K-001</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Creative Fabrica</x:v>
+      </x:c>
+      <x:c r="E3"/>
+      <x:c r="F3" t="str">
+        <x:v>Greenhouse / Reddit</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>https://job-boards.eu.greenhouse.io/creativefabrica/jobs/4807276101</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Ecommerce / marketing ops</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Needs AI workflows for email operations, content pipelines, campaign execution, optimization, and HITL governance</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>qualified</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>Prepare application package; submission needs resume/CV, LinkedIn URL, city, and AI marketing tool list</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>Recent public job post; high relevance but requires personal application details</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>C10K-002</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>GCS</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>mohammed.k@gc-ti.com</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Public hiring email</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>https://community.n8n.io/t/hiring-we-are-looking-for-a-n8n-automation-expert-to-build-ai-agent-workflows-freelance/132551</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>AI workflow / document automation</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Asked for n8n multi-agent workflow developer to ingest and analyze documents and generate downstream AI prompts</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>ready_to_contact</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Send concise contractor-trial application with live demo link and no inflated credentials</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>Older post but direct application email and relevant scope</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>C10K-003</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Talents Team</x:v>
+      </x:c>
+      <x:c r="E5"/>
+      <x:c r="F5" t="str">
+        <x:v>Make Community</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>https://community.make.com/t/hiring-make-com-http-make-com-automation-engineer-contract-part-time/103508</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Automation contractor</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Needs Make scenarios, routers, scheduling, error handling, APIs, data mapping, docs, troubleshooting</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>Workflow Triage</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>qualified</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>Apply via Make Community DM if account access is available</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>No direct email visible; avoid scraping or bypassing platform</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>C10K-004</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Creative Fabrica Reddit poster</x:v>
+      </x:c>
+      <x:c r="E6"/>
+      <x:c r="F6" t="str">
+        <x:v>Reddit</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1t49b3r/hiring_ai_marketing_specialist_agentic_ai/</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>B2C marketing automation</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Poster confirmed freelancers may be considered if similar timezone and experience at needed scale</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Workflow Triage</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>qualified</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>2026-05-08</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Use official Greenhouse application rather than unsolicited DM</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>Do not message via bots or scraped contact data</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record first Codex10k outreach
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R29c6dd2279624948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4331feac32f443dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R24c822c27ce34002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R45518841e17d4c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra1496c41dbe44b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4331941d22134198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2d3a6b4ba3974b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rf6ae5f6726274eb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -579,22 +579,22 @@
         <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>ready_to_contact</x:v>
+        <x:v>contacted</x:v>
       </x:c>
       <x:c r="L4" t="str">
         <x:v>2026-05-08</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>Send concise contractor-trial application with live demo link and no inflated credentials</x:v>
+        <x:v>Watch for reply; if positive, request anonymized sample docs and scope paid triage</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>2026-05-09</x:v>
+        <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>docs/opportunity-log.md</x:v>
+        <x:v>gmail:19e08e41f4d7c336</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>Older post but direct application email and relevant scope</x:v>
+        <x:v>Sent from Codex10k pipeline with labels Codex10k/Lead and Codex10k/Sent</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
Pivot Codex10k to fixed-scope client delivery
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra1496c41dbe44b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4331941d22134198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2d3a6b4ba3974b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rf6ae5f6726274eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4d5e9b0fe3374d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R1712d5e1507343c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R396de87b6db74e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R179c26beb4874937"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTA(Prospects!A2:A200)</x:f>
-        <x:v>5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -529,13 +529,13 @@
         <x:v>Workflow Revenue Recovery Sprint</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>qualified</x:v>
+        <x:v>hold_employment_style</x:v>
       </x:c>
       <x:c r="L3" t="str">
         <x:v>2026-05-08</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>Prepare application package; submission needs resume/CV, LinkedIn URL, city, and AI marketing tool list</x:v>
+        <x:v>Do not apply as a job; pursue only if a fixed-scope vendor/project contact path appears</x:v>
       </x:c>
       <x:c r="N3" t="str">
         <x:v>2026-05-09</x:v>
@@ -544,7 +544,7 @@
         <x:v>docs/opportunity-log.md</x:v>
       </x:c>
       <x:c r="P3" t="str">
-        <x:v>Recent public job post; high relevance but requires personal application details</x:v>
+        <x:v>Recent public job post but requires personal application details and likely employee-style involvement</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -579,7 +579,7 @@
         <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>contacted</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L4" t="str">
         <x:v>2026-05-08</x:v>
@@ -591,10 +591,10 @@
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>gmail:19e08e41f4d7c336</x:v>
+        <x:v>gmail:19e08e71637b72c1</x:v>
       </x:c>
       <x:c r="P4" t="str">
-        <x:v>Sent from Codex10k pipeline with labels Codex10k/Lead and Codex10k/Sent</x:v>
+        <x:v>Clarified this is not employment; Codex10k offers a done-for-you fixed-scope build</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -675,13 +675,13 @@
         <x:v>Workflow Triage</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>qualified</x:v>
+        <x:v>hold_employment_style</x:v>
       </x:c>
       <x:c r="L6" t="str">
         <x:v>2026-05-08</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>Use official Greenhouse application rather than unsolicited DM</x:v>
+        <x:v>Do not apply as job; only pursue if vendor/project path appears</x:v>
       </x:c>
       <x:c r="N6" t="str">
         <x:v>2026-05-09</x:v>
@@ -691,6 +691,206 @@
       </x:c>
       <x:c r="P6" t="str">
         <x:v>Do not message via bots or scraped contact data</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>C10K-005</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Callee AI Solutions</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>CalleeAIsolutions@gmail.com</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>https://www.skool.com/brendan/hiring-n8n-automation-engineer</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Voice AI agency automation</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Agency has client surge and needs n8n/API automation layer for bookings, outreach, lead gen, and internal ops</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>Watch for reply; if positive, request anonymized input/output and scope paid milestone</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>gmail:19e08eb2da5715f2</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>Sent done-for-you fixed-scope build offer; no employee-role framing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>C10K-006</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Strive Digital</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>bruno@strive-digital.com</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>LinkedIn public post</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>https://br.linkedin.com/company/strivedigitall</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Outbound lead-gen / data ops</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Needs main database plus per-client sheet workflow with duplicate prevention and client-specific statuses</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>Watch for reply; if positive, request anonymized main DB and 2 client sheets</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>gmail:19e08eb918b791a3</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>Sent fixed-scope project proposal around their exact data synchronization problem</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>C10K-007</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Bluestork AI</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>contact.bluestork.ai@gmail.com</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Reddit public post</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1nnhboj</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>AI floor-plan workflow</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>Wants n8n workflow for contractors to upload floor plans and receive structured room/surface measurements</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Watch for reply; if positive, request 2-3 anonymized floor plans and target output format</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>gmail:19e08ebf205599ce</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>Sent fixed-scope milestone offer for upload/extraction/review/output workflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>C10K-008</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Shilling Strategy Consulting</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>keerthivasan@shillingstrategyconsulting.com</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>LinkedIn public post</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>https://in.linkedin.com/company/shilling-strategy-consulting-ssc</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Consulting / workflow automation</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Public post asked for N8N automation freelancer with workflow integrations and scalable automation systems</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Watch for reply; if positive, request one workflow plus 5-10 sample records/screenshots</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>gmail:19e08ec44f776529</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>Sent done-for-you fixed-scope build offer with demo link</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Send Codex10k outreach batch
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4d5e9b0fe3374d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R1712d5e1507343c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R396de87b6db74e17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R179c26beb4874937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re3435308681642a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4f6b369aac5243cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rdb21c02757e84bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R45cc8b3e51ed4fb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTA(Prospects!A2:A200)</x:f>
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -893,6 +893,206 @@
         <x:v>Sent done-for-you fixed-scope build offer with demo link</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>C10K-009</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>RestaurantFlow OS</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>heldermiranda96@gmail.com</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>https://community.n8n.io/t/hiring-automation-engineer-wanted-n8n-core-role-restaurant-tech-startup/292053</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Restaurant revenue automation</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Needs production n8n workflows for OpenTable/SevenRooms booking data, Supabase, GHL, Printnode, multi-tenant idempotency, HMAC validation, and error handling</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Fixed-scope RestaurantFlow workflow build</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Watch for reply; if positive, request smallest workflow group, payload examples, and Supabase table shape</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>gmail:19e08f2811f81844</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>Sent USD 2500 fixed first-workflow-group offer; framed around test environment and acceptance checks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>C10K-010</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>SPAudio</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>tech@spaudio.it</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>https://community.n8n.io/t/seeking-experienced-freelance-n8n-automation-expert/207669</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Audio / operational automation</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Needs freelance support for self-hosted n8n setup, production workflows, complex API integrations, daily support, and optimization</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>n8n stabilization sprint</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>Watch for reply; if positive, request top failing workflow, apps/APIs involved, and hosting mode</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>gmail:19e08f2a422b2929</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>Sent USD 1800 fixed stabilization package offer for one priority workflow/integration plus operator guide</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>C10K-011</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>PristinePro Technologies</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>careers@pristineprotech.com</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Reddit public post / company site</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1p03o0g/looking_for_n8n_developer_with_2_years_of/</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>AI automation consultancy</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Public post asked for n8n AI agent help; company site shows AI automation work around transcription, media processing, and document updates</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Fixed-scope n8n AI agent build</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>Watch for reply; if positive, request one workflow and 5-10 anonymized sample records/screenshots</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>gmail:19e08f2c2d25180a</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>Sent USD 1500-2500 fixed workflow offer; no employee-role framing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>C10K-012</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Noevo</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>io@noevo.io</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>LinkedIn public post / company site</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>https://lk.linkedin.com/jobs/view/n8n-%2B-ai-automation-assistant-part-time-at-noevo-io-4347043760</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>EdTech operations automation</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Public posting described n8n and AI automation needs for AI-powered student counselor platform; site shows application support and document checklist workflows</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Fixed-scope Noevo operations workflow build</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>Watch for reply; if positive, request one workflow and anonymized input/output examples</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>gmail:19e08f2e136045e9</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>Sent USD 1500 fixed workflow offer for intake, checklist, routing, reminders, or reporting</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Send Codex10k specialized outreach
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re3435308681642a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4f6b369aac5243cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rdb21c02757e84bfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R45cc8b3e51ed4fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R394137368f8444d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R7d98749983f84c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Reb06f0257d954f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rc931d799d34c47db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTA(Prospects!A2:A200)</x:f>
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1093,6 +1093,156 @@
         <x:v>Sent USD 1500 fixed workflow offer for intake, checklist, routing, reminders, or reporting</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>C10K-013</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>MJBLAW</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>jshenkar@bernllp.com</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>https://community.n8n.io/t/law-firm-is-looking-for-fractional-support-in-n8n/264725</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Legal operations automation</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>Law firm asked for fractional support developing and maintaining Monday.com workflows, n8n automations, operational efficiency, and integration projects</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Fixed-scope Monday.com + n8n legal-ops workflow</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Watch for reply; if positive, request one manual/fragile workflow, Monday.com board structure, and anonymized records</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>gmail:19e08fa5b32c3037</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>Sent USD 1500-2500 fixed one-workflow offer with confidentiality and data-minimization framing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>C10K-014</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>BoviC</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>borhanovic11@gmail.com</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>https://community.n8n.io/t/looking-for-n8n-expert-accounting-automation-saudi-vat/264293</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Accounting automation</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>Asked for n8n expert to build Saudi VAT accounting automation system</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Fixed-scope accounting ingestion-to-review workflow</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>Watch for reply; if positive, require approved VAT rules, anonymized samples, and explicit no tax/legal advice boundary</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>gmail:19e08fa8fbc3903d</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>Sent USD 2500 fixed technical automation milestone; stated Codex will not certify tax/ZATCA compliance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>C10K-015</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>El Wong AI startup</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>elwongyvr@gmail.com</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>https://community.n8n.io/t/now-hiring-operations-pm-for-ai-startup/294087</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Startup operations automation</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Fast-growing AI startup needs delivery, onboarding, team coordination, process docs, systems audits, and implementation plans around Notion, Airtable, and ClickUp</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Fixed-scope ops workflow build</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>Watch for reply; if positive, request one onboarding/delivery workflow and anonymized input/output examples</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>gmail:19e08faaff62fd56</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>Sent USD 1500 fixed implementation slice offer; explicitly not a full-time PM application</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Send additional Codex10k outreach
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R394137368f8444d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R7d98749983f84c05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Reb06f0257d954f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rc931d799d34c47db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R603d547a8b1844e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R70270e0187b94dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R6ca2d374834b487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0d10a313762c4067"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -285,8 +285,8 @@
         <x:v>Qualified Prospects</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:f>COUNTA(Prospects!A2:A200)</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -294,7 +294,7 @@
         <x:v>Interested Prospects</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:f>COUNTIF(Prospects!G2:G200,"Interested")</x:f>
+        <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -975,22 +975,20 @@
         <x:v>n8n stabilization sprint</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>contacted_fixed_scope</x:v>
+        <x:v>bounced</x:v>
       </x:c>
       <x:c r="L12" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M12" t="str">
-        <x:v>Watch for reply; if positive, request top failing workflow, apps/APIs involved, and hosting mode</x:v>
-      </x:c>
-      <x:c r="N12" t="str">
-        <x:v>2026-05-11</x:v>
-      </x:c>
+        <x:v>Do not retry tech@spaudio.it; find alternate official SPAudio contact only if public and relevant</x:v>
+      </x:c>
+      <x:c r="N12"/>
       <x:c r="O12" t="str">
-        <x:v>gmail:19e08f2a422b2929</x:v>
+        <x:v>gmail:19e08f2ac74d0895</x:v>
       </x:c>
       <x:c r="P12" t="str">
-        <x:v>Sent USD 1800 fixed stabilization package offer for one priority workflow/integration plus operator guide</x:v>
+        <x:v>Original send gmail:19e08f2a422b2929 bounced with 550 5.1.1 address not found</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1241,6 +1239,456 @@
       </x:c>
       <x:c r="P17" t="str">
         <x:v>Sent USD 1500 fixed implementation slice offer; explicitly not a full-time PM application</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>C10K-016</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Aditya Das AI agency</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>aditya.das.own@gmail.com</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>https://www.skool.com/%40aditya-das-5910?g=ai-automation-society</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>AI agency / voice + CRM automation</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>Recent post asked for a single long-term n8n, Vapi, and GoHighLevel partner with live project proof</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>Fixed-scope n8n/Vapi/GHL workflow build</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>Watch for reply; if positive, request one client workflow, current GHL/Vapi stack, and sample payloads</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>gmail:19e09038c416fd10</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>Sent USD 1800 fixed first workflow group offer; framed as implementation partner, not employee application</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>C10K-017</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Mattia Tessaro / AI products</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>ecomaichatbot@gmail.com</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>https://www.skool.com/ai-automation-society/were-hiring-freelance-ai-developer-start-immediately-2?p=1c7ac68c</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>AI product / chatbot automation</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>Post requested a freelance AI developer for custom chatbots, AI agents, n8n or Voiceflow workflows, and practical shipped proof</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>Fixed-scope AI agent or n8n task build</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>Watch for reply; if positive, ask for one task, target stack, and definition of done</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>gmail:19e0903b1170799f</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>Sent USD 1200-1800 fixed first task offer with demo link</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>C10K-018</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Krishna Aggarwal</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>talktokrishna321@gmail.com</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>https://www.skool.com/%40f2fb6908044349598d33f95bdad887f1?g=5minai-2861</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>AI workflow collaboration</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Public post asked for a n8n developer to collaborate on smart automations and AI-powered workflows; profile is recently active</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>Fixed-scope n8n automation collaboration</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>Watch for reply; if positive, request apps involved, current manual steps, and desired output</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>gmail:19e0903cedbdd1bf</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>Sent USD 1200-2000 fixed workflow group offer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>C10K-019</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Peernation / KnowledgeIQ</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>bob@peernation.co</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>https://community.n8n.io/t/looking-for-experience-n8n-builder-1-to-2-years-experience/245570</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Platform workflow automation</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>Public n8n post asked builders to email Bob for platform workflow development with hands-on n8n experience</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>Fixed-scope platform workflow build</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>Watch for reply; if positive, ask for one workflow description, tools, and acceptance criteria</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>gmail:19e0903f1d028522</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>Sent USD 1200-1800 first milestone offer using test workspace/dummy data boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>C10K-020</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>SB CAIO / Aman Gupta</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>guptaaman060491@gmail.com; nematovjasurbek577@gmail.com</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>https://www.skool.com/seamless-8336/hiring-for-ai-automation-devs-n8n-or-makecom-experience-preferred</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>AI automation agency overflow</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>Post requested contractual AI automation specialists for n8n/Make, APIs, AI agents, and real-world business workflows</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>Fixed-scope overflow n8n/Make workflow build</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>Watch for reply; if positive, request one active client workflow, current manual process, and desired output</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O22" t="str">
+        <x:v>gmail:19e09040f45a4f6b</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>Sent USD 1200-2500 overflow project offer; explicitly framed as fixed-scope execution partner</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>C10K-021</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Elite Staffing Solutions / Wichita Staffing</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>info@wichitastaffing.com</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Make Community public post / official site</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>https://community.make.com/t/hiring-make-com-monday-com-expert-help-scale-my-staffing-business-with-smart-ai-automations/107133</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Staffing order intake automation</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>Founder asked for Make.com + Monday.com automation to parse forwarded order emails, extract details with AI, check Monday.com via GraphQL, create AutoFlow items, and alert on blocked orders</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Fixed-scope order-intake stabilization build</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>Watch for reply; if positive, request 3-5 failing order emails, Monday board fields, and successful AutoFlow item shape</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>gmail:19e0905b7db83be0</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>Sent USD 1800 fixed Order Intake v1 offer; official contact page listed info@wichitastaffing.com</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>C10K-022</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Graeham Watts / Intero Real Estate</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>graehamwatts@gmail.com</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>n8n Community public post / public real estate profile</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>https://community.n8n.io/t/looking-for-an-experienced-n8n-developer-to-help-implement-a-production-real-estate-automation-system-paid/247380</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Real estate automation</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>Public post requested paid help on production GoHighLevel + n8n + SearchAtlas real estate workflows for lead routing, follow-up, nurture, outreach, messaging, video, and calls</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>Fixed-scope GHL+n8n reliability sprint</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>Watch for reply; if positive, request highest-risk workflow, GHL trigger, success/failure behavior, and sample lead records</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
+        <x:v>gmail:19e0905d640c02d5</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>Sent USD 1800-2500 reliability milestone offer; email found on public real estate profiles/listings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>C10K-023</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>nocodecreative.io / Wayne Simpson</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>wayne@nocodecreative.io; hello@sales.nocodecreative.io</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>n8n Community public post / official site</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>https://community.n8n.io/t/we-re-hiring/247068</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Automation agency overflow</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>Public post sought contract/freelance n8n developer help; official site shows AI, low-code, API, workflow automation, and app development services</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>Fixed-scope n8n overflow build</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>Watch for reply; if positive, request client-safe brief, tools involved, and definition of done</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O25" t="str">
+        <x:v>gmail:19e0905f6b7f8fe0</x:v>
+      </x:c>
+      <x:c r="P25" t="str">
+        <x:v>Sent USD 1500-2500 fixed overflow build offer to founder and sales inbox</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>C10K-024</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Merch Club</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>jay@merchclub.com</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Reddit public post</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1q52ks7/hiringremote_skilled_n8n_workflow_automation/</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Ecommerce shipping notification automation</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>Public post asked for n8n shipping notification automation using Google Sheets, carrier APIs, OpenAI review prompts, weather, Supermail/Gmail, logging, and delay alerts</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>Fixed-scope Shipping Notification v1</x:v>
+      </x:c>
+      <x:c r="K26" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L26" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M26" t="str">
+        <x:v>Watch for reply; if positive, request sample sheet structure, example order row, preferred email service, and carrier API</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O26" t="str">
+        <x:v>gmail:19e090615f966eaf</x:v>
+      </x:c>
+      <x:c r="P26" t="str">
+        <x:v>Sent USD 1800 fixed Shipping Notification v1 offer</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Send additional Codex10k direct outreach
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R603d547a8b1844e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R70270e0187b94dcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R6ca2d374834b487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0d10a313762c4067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0a26571f8578487c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R65e95c2df7a747d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Ra5f3393a98854cf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rdec6e3a9852e4cee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>21</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1691,6 +1691,456 @@
         <x:v>Sent USD 1800 fixed Shipping Notification v1 offer</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>C10K-025</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Mcode Consulting</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>anushka@mcodehq.com</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Reddit public post</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1rxs43t/hiring_video_ai_automation_farm_for_product/</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Product video automation</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>Public post asked for a Video AI Automation Farm for product content with company, website, and email listed</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>Fixed-scope Video Automation v1</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>Watch for reply; if positive, request target video format, product input fields, preferred generation tools, and first-batch acceptance checks</x:v>
+      </x:c>
+      <x:c r="N27" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O27" t="str">
+        <x:v>gmail:19e090bef5321288</x:v>
+      </x:c>
+      <x:c r="P27" t="str">
+        <x:v>Sent USD 2500 fixed Video Automation v1 offer using dummy product data/test assets first</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>C10K-026</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Next Level Growth Partner / Tom Santella</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>tom@nextlevelgrowthpartner.com</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>https://www.skool.com/ai-automation-society/hiring-6ae4ab1f?p=b7283e18</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Agency fulfillment automation</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>Public post asked for n8n fulfillment around outreach workflows, GHL integrations, voice AI, chat widgets, and lead-conversion automations</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>Compliance-first lead-response workflow</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M28" t="str">
+        <x:v>Watch for reply; if positive, keep strict no-spam/no-deceptive-autonomy boundary and request one client-safe workflow brief</x:v>
+      </x:c>
+      <x:c r="N28" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O28" t="str">
+        <x:v>gmail:19e090c15f5b9de0</x:v>
+      </x:c>
+      <x:c r="P28" t="str">
+        <x:v>Sent USD 2500 fixed compliant lead-response/booked-call workflow offer; explicitly refused spam, deceptive impersonation, and policy-evasion flows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>C10K-027</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Arif Asgar</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>arif.askerov99@gmail.com</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Skool public post</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>https://www.skool.com/ai-automation-society/looking-for-senior-n8n-makecom-automation-expert-2-years-experience?p=bfc5565c</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Automation agency overflow</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>Public post asked for experienced n8n/Make specialist for complex custom workflows across legal, real estate, healthcare, and e-commerce</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>Fixed-scope n8n/Make overflow build</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>Watch for reply; if positive, request tools involved, current manual process, exact expected output, and acceptance checks</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O29" t="str">
+        <x:v>gmail:19e090c353941289</x:v>
+      </x:c>
+      <x:c r="P29" t="str">
+        <x:v>Sent USD 1500-2500 fixed workflow group offer; framed as overflow implementation capacity, not employee role</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>C10K-028</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>Momentum Digital</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>hi@needmomentum.com</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Glassdoor public posting</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>https://www.glassdoor.com/job-listing/gohighlevel-ghl-expert-%E2%80%93-marketing-and-sales-systems-momentum-digital-JV_KO0%2C52_KE53%2C69.htm?jl=1009934837935</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>GHL workflow systems</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>Public posting sought GoHighLevel expert for marketing and sales systems; fit as fixed-scope workflow sprint instead of full-time role</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>Fixed-scope GHL workflow sprint</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>Watch for reply; if positive, request one pipeline/client snapshot, current failure path, and acceptance checklist</x:v>
+      </x:c>
+      <x:c r="N30" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O30" t="str">
+        <x:v>gmail:19e090d9ae99fe47</x:v>
+      </x:c>
+      <x:c r="P30" t="str">
+        <x:v>Sent USD 2500 fixed 10-day GHL workflow sprint; framed as not full-time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>C10K-029</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>Gachet Ponzellini LLC</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>admin@gachetponzellini.com</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Reddit public post</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1qmbmd0/looking_for_n8n_automation_dev_ocr_parsing/</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Tax document OCR automation</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>Public post listed a USD 1200 fixed n8n OCR/parsing/Postgres project with direct email and sensitive tax-doc constraints</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Fixed-scope n8n OCR/Postgres build</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>Watch for reply only; no further outbound unless they respond because a prior separate-run message existed</x:v>
+      </x:c>
+      <x:c r="N31" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O31" t="str">
+        <x:v>gmail:19e091058299e02a</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>Sent USD 1200 fixed first-release offer with sanitized/redacted sample boundary; prior separate-run message gmail:19e08dedf46b363f found after send</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>C10K-030</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>Bendito Soft Tech Pvt Ltd</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>contact@benditosofttech.com</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>LinkedIn/Glassdoor public posting</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>https://in.linkedin.com/jobs/view/senior-ghl-automation-ai-developer-at-bendito-soft-tech-pvt-ltd-4406932933</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>GHL agency delivery overflow</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>Public posting asked for GHL snapshots, CRM pipelines, workflows, email/SMS automation, webhooks, Make/Zapier, DNS/email setup, and AI-assisted debugging</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>Fixed-scope GHL/AI automation pilot</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M32" t="str">
+        <x:v>Watch for reply; if positive, request one client-safe snapshot/workflow brief and define test-subaccount access</x:v>
+      </x:c>
+      <x:c r="N32" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O32" t="str">
+        <x:v>gmail:19e091083db2bcb0</x:v>
+      </x:c>
+      <x:c r="P32" t="str">
+        <x:v>Sent USD 1500 fixed 5-business-day overflow pilot; no live client data until access boundaries agreed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>C10K-031</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>Terborg Zorg</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>info@terborgzorg.nl</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Reddit public post / official contact page</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1sti7jh/automation_expert_wanted/</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>Healthcare recruitment automation</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>Public post asked for automation ownership across Meta Ads, n8n, Supabase, GoHighLevel, Bendy, Otentica, and Claude AI from ad click to signed contract</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>GDPR-safe n8n/GHL/Supabase hardening sprint</x:v>
+      </x:c>
+      <x:c r="K33" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L33" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>Watch for reply; if positive, request anonymized workflow map/screenshots and the highest-failure handoff only</x:v>
+      </x:c>
+      <x:c r="N33" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O33" t="str">
+        <x:v>gmail:19e0910ab68fecff</x:v>
+      </x:c>
+      <x:c r="P33" t="str">
+        <x:v>Sent USD 2500 7-day hardening sprint offer; explicitly no candidate, patient, or contract data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>C10K-032</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>Swoopa / Rory</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>rory@getswoopa.com</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>https://community.n8n.io/t/we-are-looking-for-someone-who-has-experience-with-n8n-and-ghl/279268</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>SaaS lead/support/trial follow-up</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>Public post asked for help making sure no lead, support request, or trial user is left without follow-up across GHL, OpenPhone, Gmail, and workflow systems</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>Fixed-scope n8n + GHL reliability sprint</x:v>
+      </x:c>
+      <x:c r="K34" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L34" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M34" t="str">
+        <x:v>Watch for reply; if positive, request the single follow-up path leaking the most value plus anonymized payloads/test account</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O34" t="str">
+        <x:v>gmail:19e0911955a5ca92</x:v>
+      </x:c>
+      <x:c r="P34" t="str">
+        <x:v>Sent USD 2500 fixed stabilized workflow group offer with test-contact and no-customer-data boundary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>C10K-033</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>GoodieX Tech LLC</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>admin@goodiex-tech.com</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>Reddit public post / official site</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>https://www.reddit.com/r/n8n/comments/1r69egp/looking_for_n8n_automation_expert/</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>Clothing sales lifecycle automation</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>Public post requested an n8n automation expert to manage the full sales lifecycle for a clothing business</x:v>
+      </x:c>
+      <x:c r="J35" t="str">
+        <x:v>Fixed-scope n8n sales-lifecycle sprint</x:v>
+      </x:c>
+      <x:c r="K35" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L35" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M35" t="str">
+        <x:v>Watch for reply; if positive, request one highest-manual sales step, sample order/customer shape, and preferred messaging channel</x:v>
+      </x:c>
+      <x:c r="N35" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O35" t="str">
+        <x:v>gmail:19e0911b9155643c</x:v>
+      </x:c>
+      <x:c r="P35" t="str">
+        <x:v>Sent USD 1800 fixed first workflow sprint; dummy/test customers only and simple labels for Spanish translation</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Advance Codex10k interested deal tracking
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0a26571f8578487c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R65e95c2df7a747d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Ra5f3393a98854cf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rdec6e3a9852e4cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8006b7452b6542f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rde80db0734be4e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Red074f1608604dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Re52e0a1e2f1c479f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -294,8 +294,8 @@
         <x:v>Interested Prospects</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"interested_phase0_sent") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -822,25 +822,25 @@
         <x:v>Wants n8n workflow for contractors to upload floor plans and receive structured room/surface measurements</x:v>
       </x:c>
       <x:c r="J9" t="str">
-        <x:v>10-Day Workflow Revenue Recovery Sprint</x:v>
+        <x:v>Paid floor-plan feasibility milestone</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>contacted_fixed_scope</x:v>
+        <x:v>interested_phase0_sent</x:v>
       </x:c>
       <x:c r="L9" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>Watch for reply; if positive, request 2-3 anonymized floor plans and target output format</x:v>
+        <x:v>Wait for sample floor plans or meeting-link reply; if they accept, send invoice/payment link for USD 1200 Phase 0</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>2026-05-11</x:v>
+        <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>gmail:19e08ebf205599ce</x:v>
+        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Sent fixed-scope milestone offer for upload/extraction/review/output workflow</x:v>
+        <x:v>Inbound reply asked for online meeting and noted floor-plan variation complexity; sent USD 1200 Phase 0 feasibility offer credited toward USD 4500-7500 implementation</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2139,6 +2139,106 @@
       </x:c>
       <x:c r="P35" t="str">
         <x:v>Sent USD 1800 fixed first workflow sprint; dummy/test customers only and simple labels for Spanish translation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>C10K-034</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>Town of Duck NC</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>knickens@ducknc.gov</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>https://ducknc.gov/news/request-for-proposals-website-redesign-cms-implementation/</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>Municipal website CMS QA</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>Public RFP requested comprehensive website redesign and CMS implementation with proposal deadline May 14 2026</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>Accessibility/CMS workflow QA support option</x:v>
+      </x:c>
+      <x:c r="K36" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L36" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M36" t="str">
+        <x:v>Watch for procurement reply; if positive, send one-page scope and acceptance checklist for USD 6500 support option</x:v>
+      </x:c>
+      <x:c r="N36" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O36" t="str">
+        <x:v>gmail:19e0918f02a759bd</x:v>
+      </x:c>
+      <x:c r="P36" t="str">
+        <x:v>Sent USD 6500 10-business-day accessibility/CMS QA support option; explicitly not a prime full-service municipal redesign-firm submission</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>C10K-035</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Hunger Task Force</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>zachary@hungertaskforce.org</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>https://www.hungertaskforce.org/2026/03/18/website-redesign-rfp/</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>Nonprofit website/donation workflow QA</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>Public RFP described full website rebuild focused on food-resource access, monthly recurring donations, WCAG 2.1 AA, and Blackbaud/Fundraise Up/Quorum/Galaxy integrations; proposal deadline passed but vendor selection listed May 20 2026</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>Donation/accessibility launch QA support option</x:v>
+      </x:c>
+      <x:c r="K37" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L37" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M37" t="str">
+        <x:v>Watch for reply; if positive, request CMS/integration stack and send one-page scope with acceptance criteria</x:v>
+      </x:c>
+      <x:c r="N37" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O37" t="str">
+        <x:v>gmail:19e0919708d02b01</x:v>
+      </x:c>
+      <x:c r="P37" t="str">
+        <x:v>Sent USD 9000 donation/accessibility/workflow QA support option for internal team or selected vendor; no donor/client/beneficiary data by email</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Send Codex10k launch QA outreach
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8006b7452b6542f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rde80db0734be4e5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Red074f1608604dfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Re52e0a1e2f1c479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5242671a734545b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R3ac40232798844bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Ra42109027e4c4e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R1917d605a2684b15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>32</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -837,10 +837,10 @@
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360</x:v>
+        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360; gmail:19e09217059048e0</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Inbound reply asked for online meeting and noted floor-plan variation complexity; sent USD 1200 Phase 0 feasibility offer credited toward USD 4500-7500 implementation</x:v>
+        <x:v>Inbound reply asked for online meeting and noted floor-plan variation complexity; sent USD 1200 Phase 0 feasibility offer credited toward USD 4500-7500 implementation; then sent synthetic proof link at /#floorplan</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2239,6 +2239,106 @@
       </x:c>
       <x:c r="P37" t="str">
         <x:v>Sent USD 9000 donation/accessibility/workflow QA support option for internal team or selected vendor; no donor/client/beneficiary data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>C10K-036</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Idaho Forest Restoration Partnership</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>russ7024@vandals.uidaho.edu; idahoforestpartners@gmail.com</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>https://idahoforestpartners.org/services</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>Nonprofit website beta launch QA</x:v>
+      </x:c>
+      <x:c r="I38" t="str">
+        <x:v>Public RFP showed beta testing May 7-15 2026, final website launch June 1 2026, SiteKreator migration, resource library, redirects, accessibility, Aweber, donations/sponsorship CTAs, and staff training</x:v>
+      </x:c>
+      <x:c r="J38" t="str">
+        <x:v>Website beta QA launch-support sprint</x:v>
+      </x:c>
+      <x:c r="K38" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L38" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M38" t="str">
+        <x:v>Watch for reply; if positive, request beta/staging URL, selected CMS, resource-library status, and migration inventory</x:v>
+      </x:c>
+      <x:c r="N38" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O38" t="str">
+        <x:v>gmail:19e09231a31216c8</x:v>
+      </x:c>
+      <x:c r="P38" t="str">
+        <x:v>Sent USD 6500 7-10 business day migration/accessibility/resource-library launch QA support option; not a late replacement proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>C10K-037</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>City of Waverly IA</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>jljohnson@waverlyia.com</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>https://www.waverlyia.com/news/city-of-waverly/city-of-waverly-w.aspx</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>Municipal website launch QA</x:v>
+      </x:c>
+      <x:c r="I39" t="str">
+        <x:v>Public RFP requested website redesign, development, hosting, and maintenance services with accessible, user-friendly, sustainable platform goals; proposal deadline already passed</x:v>
+      </x:c>
+      <x:c r="J39" t="str">
+        <x:v>Website redesign launch QA support option</x:v>
+      </x:c>
+      <x:c r="K39" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L39" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M39" t="str">
+        <x:v>Watch for reply; if positive, request current project/vendor status, staging timing, CMS, and priority citizen paths</x:v>
+      </x:c>
+      <x:c r="N39" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O39" t="str">
+        <x:v>gmail:19e09234c800d9d4</x:v>
+      </x:c>
+      <x:c r="P39" t="str">
+        <x:v>Sent USD 6500 7-10 business day accessibility/CMS/migration launch QA support option; explicitly not a late full redesign proposal</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update Bluestork BygAI opportunity scope
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5242671a734545b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R3ac40232798844bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Ra42109027e4c4e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R1917d605a2684b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7eeae2664d8b448f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0be9547583814cfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2184a7e2876646ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R3738bc92ad4843ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -294,7 +294,7 @@
         <x:v>Interested Prospects</x:v>
       </x:c>
       <x:c r="B9" t="n">
-        <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"interested_phase0_sent") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
+        <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"interested_phase0_sent") + COUNTIF(Prospects!K2:K200,"meeting_proposed_phase0") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -804,43 +804,43 @@
         <x:v>Codex10k</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>Bluestork AI</x:v>
+        <x:v>Bluestork AI / BygAI.dk</x:v>
       </x:c>
       <x:c r="E9" t="str">
         <x:v>contact.bluestork.ai@gmail.com</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>Reddit public post</x:v>
+        <x:v>Reddit public post / inbound Gmail</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>https://www.reddit.com/r/n8n/comments/1nnhboj</x:v>
+        <x:v>https://bygai.dk</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>AI floor-plan workflow</x:v>
+        <x:v>Computer-vision automation lift for floor-plan measurement</x:v>
       </x:c>
       <x:c r="I9" t="str">
-        <x:v>Wants n8n workflow for contractors to upload floor plans and receive structured room/surface measurements</x:v>
+        <x:v>Buyer says BygAI.dk already has a semi-automatic solution for AI-driven floor-plan measurement to painter quote, but further computer-vision automation may be valuable; prior DTU master's student work did not generalize consistently across varied plans</x:v>
       </x:c>
       <x:c r="J9" t="str">
-        <x:v>Paid floor-plan feasibility milestone</x:v>
+        <x:v>Paid computer-vision feasibility milestone</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>interested_phase0_sent</x:v>
+        <x:v>meeting_proposed_phase0</x:v>
       </x:c>
       <x:c r="L9" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>Wait for sample floor plans or meeting-link reply; if they accept, send invoice/payment link for USD 1200 Phase 0</x:v>
+        <x:v>Wait for meeting window or link; if they engage, convert call into USD 1200 paid Phase 0 around current BygAI bottleneck and 2 anonymized examples</x:v>
       </x:c>
       <x:c r="N9" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360; gmail:19e09217059048e0</x:v>
+        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360; gmail:19e09217059048e0; gmail:19e0923670fd29ae; gmail:19e0924dd475b380</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Inbound reply asked for online meeting and noted floor-plan variation complexity; sent USD 1200 Phase 0 feasibility offer credited toward USD 4500-7500 implementation; then sent synthetic proof link at /#floorplan</x:v>
+        <x:v>Inbound reply corrected scope: existing semi-automatic product at BygAI.dk and interest only if computer vision can automate further; sent realistic meeting reply with no full-generalization promise and two Monday CEST windows</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>

<commit_message>
Send fresh Codex10k outreach batch
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7eeae2664d8b448f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0be9547583814cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2184a7e2876646ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R3738bc92ad4843ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R282339bf2b4749ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0a277ea2848549dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R97f6d45bd01f4f77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rb7eb411a295b4530"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>34</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2341,6 +2341,406 @@
         <x:v>Sent USD 6500 7-10 business day accessibility/CMS/migration launch QA support option; explicitly not a late full redesign proposal</x:v>
       </x:c>
     </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>C10K-038</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>Chain Reaction Motorcycle School</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>luke@chainreactionmotorcycleschool.com</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>Reddit public post / official site</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>https://www.reddit.com/r/AiAutomations/comments/1s599vw/looking_for_ai_automation_expert_to_build/</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>Scheduling/payment automation</x:v>
+      </x:c>
+      <x:c r="I40" t="str">
+        <x:v>Public post requested AI digital front office across Wix forms, Gmail, Stripe, Airtable, Make/Zapier, phone/SMS/email, scheduling, payments, enrollment tracking, and MSF eCourse timing</x:v>
+      </x:c>
+      <x:c r="J40" t="str">
+        <x:v>Phase 1 scheduling/payment source-of-truth build</x:v>
+      </x:c>
+      <x:c r="K40" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L40" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M40" t="str">
+        <x:v>Watch for reply; if positive, request workflow video or 3 anonymized examples and scope paid Phase 1</x:v>
+      </x:c>
+      <x:c r="N40" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O40" t="str">
+        <x:v>gmail:19e092dbf9996651</x:v>
+      </x:c>
+      <x:c r="P40" t="str">
+        <x:v>Sent USD 3500 Phase 1 offer; no student data by email; no promise of MSF RES browser automation before access review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>C10K-039</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>Ferncliff Camp and Conference Center</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>kimberly@ferncliff.org; info@ferncliff.org</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>https://ferncliff.org/about/jobs/rfps/</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>Nonprofit website launch QA</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
+        <x:v>Open website redesign RFP with May 25 proposal deadline; scope includes CampBrain, DonorPerfect, Constant Contact, ADP, Square, content migration, staff editing, accessibility, giving, camp, retreat, nature school, outreach, and store paths</x:v>
+      </x:c>
+      <x:c r="J41" t="str">
+        <x:v>Donation/integration/accessibility QA support</x:v>
+      </x:c>
+      <x:c r="K41" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L41" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>Watch for reply; if positive, send one-page acceptance checklist for support slice or selected vendor</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O41" t="str">
+        <x:v>gmail:19e092de4305b72a</x:v>
+      </x:c>
+      <x:c r="P41" t="str">
+        <x:v>Sent USD 4500 bounded QA/support option; not a prime redesign bid; no donor/camper/staff/applicant data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>C10K-040</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>City of Hidden Hills CA</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>amber@hiddenhills.gov</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>https://hiddenhills.gov/city-departments/city-clerk/notice-inviting-bids-proposals-rfps/</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>Municipal website launch QA</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>Open website redesign and development services RFP due May 15; scope includes redesign, development, hosting, training, ongoing maintenance, and public-agency CMS handoff</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>Municipal accessibility/CMS migration QA support</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L42" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>Watch for reply; only communicate through designated RFP contact; if positive, send one-page QA scope</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O42" t="str">
+        <x:v>gmail:19e092e04acef122</x:v>
+      </x:c>
+      <x:c r="P42" t="str">
+        <x:v>Sent USD 6500 launch QA support option; explicitly not bypassing RFP or replacing prime vendor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>C10K-041</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>SCIDpda</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>marione@scidpda.org</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>Public RFQ page</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>https://scidpda.org/website-redesign-and-development-for-scidpda-request-for-qualifications-rfq/</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>Community nonprofit website launch QA</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>RFQ due May 13 with October 2026 launch target; site needs donations, property listings, event calendar, RFQ/RFP postings, multilingual translation, accessibility, security, staff training, and governance materials</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>Multilingual/accessibility/security launch QA support</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L43" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M43" t="str">
+        <x:v>Watch for reply; if positive, send one-page beta QA/support scope or support selected vendor</x:v>
+      </x:c>
+      <x:c r="N43" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O43" t="str">
+        <x:v>gmail:19e092e31c4c2514</x:v>
+      </x:c>
+      <x:c r="P43" t="str">
+        <x:v>Sent USD 4000 bounded support option; not a late full redesign bid; no resident/donor/applicant/tenant data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>C10K-042</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>ShelbyKY Tourism</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>mason@visitshelbyky.com; ethan@visitshelbyky.com</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>https://www.visitshelbyky.com/articles/post/request-for-proposals-website-design/</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>Tourism website migration QA</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>Open VisitShelbyKY.com redesign RFP due May 29; moving away from Simpleview/Granicus with Whereabouts CRM collaboration, accessibility, SEO/GEO, redirects, Datafy, WhatsGood, Flodesk, analytics preservation, and post-launch support</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>Tourism website QA/accessibility support package</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L44" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M44" t="str">
+        <x:v>Watch for reply; if positive, send one-page support-subcontract scope and acceptance criteria</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O44" t="str">
+        <x:v>gmail:19e092e54ededdf6</x:v>
+      </x:c>
+      <x:c r="P44" t="str">
+        <x:v>Sent USD 7500 bounded QA/accessibility support option; not a prime website proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>C10K-043</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>Bellingham Housing Authority</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>procurement@bellinghamhousing.org; Chris.Longwell@BellinghamHousing.org</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>https://bellinghamhousing.org/request-for-proposals-website-development-and-design-services/2026/04/20/</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>Housing authority website launch QA</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>Open RFP-BHA-2026-04-IT due May 27; scope includes modern accessible public site for applicants, residents, landlords, property directory, rebrand/logo, staff training, launch, and 12-month support</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>Housing authority accessibility/property-directory launch QA support</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>Watch for reply; if positive, send one-page QA scope for selected vendor or BHA acceptance testing</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O45" t="str">
+        <x:v>gmail:19e092e797f754eb</x:v>
+      </x:c>
+      <x:c r="P45" t="str">
+        <x:v>Sent USD 6500 bounded QA/accessibility support option; not a prime redesign proposal; no applicant/resident/landlord data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>C10K-044</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>City of Willow Springs MO</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>htooley@willowspringsmo.com; bhicks@willowspringsmo.com</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>Public bid page</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>https://www.willowspringsmo.com/bids.aspx?bidID=8</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>Municipal CMS/forms/accessibility QA</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>Open website redesign and content management services RFP due May 29; replacing CivicPlus with hosted CMS, forms, staff portal, agendas/minutes, document management, ADA/WCAG, future .gov transition, and staff editor guardrails</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>CMS/forms/accessibility acceptance testing support</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L46" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M46" t="str">
+        <x:v>Watch for reply; if positive, send one-page acceptance testing scope</x:v>
+      </x:c>
+      <x:c r="N46" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O46" t="str">
+        <x:v>gmail:19e092e9eef4b373</x:v>
+      </x:c>
+      <x:c r="P46" t="str">
+        <x:v>Sent USD 6800 bounded QA/support package; not a full prime website proposal; no sensitive resident/employee/utility/payment data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>C10K-045</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>Yolo-Solano Air Quality Management District</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>BJamros@ysaqmd.org</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>https://www.ysaqmd.org/about-the-district/announcements/</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>Air district website accessibility QA</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>Open RFP for Website Redesign and Development Services with ADA Accessibility Compliance due June 1; scope includes content migration, staff training, accessibility documentation, testing, and deployment</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>Accessibility and launch QA support option</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>Watch for reply; if positive, send one-page acceptance checklist for YSAQMD or selected vendor</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O47" t="str">
+        <x:v>gmail:19e092ebf47ff420</x:v>
+      </x:c>
+      <x:c r="P47" t="str">
+        <x:v>Sent USD 6500 bounded QA/accessibility support option; not a prime redesign proposal</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Send Synergy outreach and prep Visualfestation packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R282339bf2b4749ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0a277ea2848549dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R97f6d45bd01f4f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rb7eb411a295b4530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R072587d7c1394be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R9c9221ba3c234948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R0dd0e55a460f4693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rec0d5b5feac64c6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>42</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -295,7 +295,7 @@
       </x:c>
       <x:c r="B9" t="n">
         <x:f>COUNTIF(Prospects!K2:K200,"interested") + COUNTIF(Prospects!K2:K200,"interested_phase0_sent") + COUNTIF(Prospects!K2:K200,"meeting_proposed_phase0") + COUNTIF(Prospects!K2:K200,"proposal_sent") + COUNTIF(Prospects!K2:K200,"invoice_sent") + COUNTIF(Prospects!K2:K200,"paid")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -825,22 +825,22 @@
         <x:v>Paid computer-vision feasibility milestone</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>meeting_proposed_phase0</x:v>
+        <x:v>phase0_reply_sent_awaiting_approval</x:v>
       </x:c>
       <x:c r="L9" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>Wait for meeting window or link; if they engage, convert call into USD 1200 paid Phase 0 around current BygAI bottleneck and 2 anonymized examples</x:v>
+        <x:v>Wait for Bluestork to confirm Tuesday May 12 meeting time or approve USD 1200 Phase 0; if approved, prepare payment link/invoice and record settlement evidence before ledger credit</x:v>
       </x:c>
       <x:c r="N9" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360; gmail:19e09217059048e0; gmail:19e0923670fd29ae; gmail:19e0924dd475b380</x:v>
+        <x:v>gmail:19e091525a4d297b; gmail:19e0916f642c7360; gmail:19e09217059048e0; gmail:19e0923670fd29ae; gmail:19e0924dd475b380; gmail:19e094216cbfaeeb; gmail:19e09449bd7d27aa; private/bluestork/bluestork_phase0_proof.md; docs/bluestork-phase0-scope.md; outputs/codex10k/bluestork-phase0-scope.pdf; gmail:19e0af07c7a8730e; docs/bluestork-phase0-payment-request.md; outputs/codex10k/bluestork-phase0-payment-request-draft.pdf</x:v>
       </x:c>
       <x:c r="P9" t="str">
-        <x:v>Inbound reply corrected scope: existing semi-automatic product at BygAI.dk and interest only if computer vision can automate further; sent realistic meeting reply with no full-generalization promise and two Monday CEST windows</x:v>
+        <x:v>Sent in-thread reply with public-safe Phase 0 scope PDF attached. Reply accepted Tuesday May 12 at 11:00 Danish time, positioned the three PDFs as suitable Phase 0 samples, recommended USD 1200 Phase 0, and requested wall-height/opening-deduction rules before final net wall-area claims. Prepared payment request draft and estimated processor-fee math for immediate invoice/payment-link step after approval.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2123,22 +2123,22 @@
         <x:v>Fixed-scope n8n sales-lifecycle sprint</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>contacted_fixed_scope</x:v>
+        <x:v>intro_video_sent_awaiting_response</x:v>
       </x:c>
       <x:c r="L35" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M35" t="str">
-        <x:v>Watch for reply; if positive, request one highest-manual sales step, sample order/customer shape, and preferred messaging channel</x:v>
+        <x:v>Wait for GoodieX to send current tools and the highest-friction sales step; if positive prepare Stripe Payment Link or hosted invoice for USD 1800 v1 scope</x:v>
       </x:c>
       <x:c r="N35" t="str">
-        <x:v>2026-05-11</x:v>
+        <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>gmail:19e0911b9155643c</x:v>
+        <x:v>gmail:19e0911b9155643c; gmail:19e0d8f21a4d07e1; gmail:19e0dbc2e35630dc; goodiex-intro.html; outputs/codex10k/goodiex-n8n-sales-lifecycle-blueprint.json; docs/goodiex-intro-video-script.md; docs/goodiex-v1-scope.md</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>Sent USD 1800 fixed first workflow sprint; dummy/test customers only and simple labels for Spanish translation</x:v>
+        <x:v>Krystal Boyd replied asking for an introduction video. User approved the response and Gmail reply 19e0dbc2e35630dc sent the client-facing intro walkthrough link; sample n8n blueprint added to the public page; payment-ready USD 1800 v1 scope is prepared but not sent.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2673,22 +2673,22 @@
         <x:v>CMS/forms/accessibility acceptance testing support</x:v>
       </x:c>
       <x:c r="K46" t="str">
-        <x:v>contacted_fixed_scope</x:v>
+        <x:v>identity_clarified_awaiting_review</x:v>
       </x:c>
       <x:c r="L46" t="str">
         <x:v>2026-05-09</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>Watch for reply; if positive, send one-page acceptance testing scope</x:v>
+        <x:v>Wait for City review after bids are submitted; if they ask for more detail, send one-page USD 6800 QA/accessibility acceptance-testing scope</x:v>
       </x:c>
       <x:c r="N46" t="str">
         <x:v>2026-05-14</x:v>
       </x:c>
       <x:c r="O46" t="str">
-        <x:v>gmail:19e092e9eef4b373</x:v>
+        <x:v>gmail:19e092e9eef4b373; gmail:19e0970a8808eef1; gmail:19e0af09f34ad913</x:v>
       </x:c>
       <x:c r="P46" t="str">
-        <x:v>Sent USD 6800 bounded QA/support package; not a full prime website proposal; no sensitive resident/employee/utility/payment data by email</x:v>
+        <x:v>Sent in-thread reply clarifying Nakul is an independent freelancer / sole proprietor, not a larger company; kept the fixed-scope support option bounded for the City or selected website vendor.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2739,6 +2739,680 @@
       </x:c>
       <x:c r="P47" t="str">
         <x:v>Sent USD 6500 bounded QA/accessibility support option; not a prime redesign proposal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>C10K-046</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>Visualfestation / Peter Adams</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>visualfestation@gmail.com</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>https://community.make.com/t/looking-to-hire-a-pro-for-integration/107978</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>Make integration</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>Public Hire a Pro post asked for help integrating Skool, Zendo, Airtable, Rewardful, and Stripe and listed direct email</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>Payment/access/affiliate integration v1</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>proposal_packet_ready_no_gmail</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>Use non-Gmail/manual-approved channel only; do not send via Gmail unless user reverses instruction</x:v>
+      </x:c>
+      <x:c r="N48"/>
+      <x:c r="O48" t="str">
+        <x:v>docs/outbox-next.md</x:v>
+      </x:c>
+      <x:c r="P48" t="str">
+        <x:v>Prepared USD 1200 fixed v1 copy; no live payment credentials by email; use Stripe test mode and least-privilege access</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>C10K-047</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>SoIN Tourism / Clark-Floyd Counties CVB</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Janelle@GoSoIN.com</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Public RFP page</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>https://www.gosoin.com/request-for-proposals/</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>Tourism CMS/CRM/partner portal launch QA</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>Open RFP for website services, CMS, CRM system of record, and Partner Portal/Extranet; questions due June 1 and proposals due July 1 2026</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>CMS/CRM/partner portal launch QA support</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>proposal_packet_ready_no_gmail</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Use non-Gmail RFP submission route or manual-approved channel; do not send via Gmail unless user reverses instruction</x:v>
+      </x:c>
+      <x:c r="N49"/>
+      <x:c r="O49" t="str">
+        <x:v>docs/outbox-next.md</x:v>
+      </x:c>
+      <x:c r="P49" t="str">
+        <x:v>Preparing USD 8500 bounded launch-QA support proposal; no individual pre-submission meeting request; no visitor/partner/CRM production data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>C10K-048</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Lindsey Moore / Make.com specialist search</x:v>
+      </x:c>
+      <x:c r="E50"/>
+      <x:c r="F50" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>https://community.make.com/t/make-com-automation-specialist-ongoing-or-project-based/107052</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>AI workflow automation / internal ops</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>Public Hire Help post from April 7, 2026 asks for an experienced Make specialist to build and maintain automations across Slack, ClickUp, Google Workspace, and Claude with monitoring, error alerts, and documentation</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Reliability-first Make build and maintenance sprint</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>Manual follow-up only if this thread is still open; lead with one production-grade Make workflow plus monitoring/alerting sample</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O50" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P50" t="str">
+        <x:v>Project-based or ~10 hours/week; strong fit for AI workflow hardening but no outreach in monitor run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>C10K-049</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>Charbel Sarkis / facilities maintenance company</x:v>
+      </x:c>
+      <x:c r="E51"/>
+      <x:c r="F51" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>https://community.make.com/t/expert-needed-google-workspace-facil-it-google-chat-work-order-intake-automation/102786</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>Lead intake / work order ops</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>U.S. facilities maintenance company says high-volume work orders arrive by email and portals and wants a Make MVP in ~30 days to parse Gmail work orders into FACIL-IT with Google Chat coordination</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>Work-order intake and triage MVP</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Manual follow-up only; angle should be bounded Gmail-to-system intake with idempotency, parsing confidence checks, and escalation path</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O51" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P51" t="str">
+        <x:v>Directly matches intake automation pain and has a concrete 30-day MVP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>C10K-050</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>JR Pool Pros / Jose Rodriguez</x:v>
+      </x:c>
+      <x:c r="E52"/>
+      <x:c r="F52" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>https://community.make.com/t/automations-with-api-jobtread-voiceflow-and-airtable/104131</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>Quote/workflow memory automation</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>Owner describes 40 active pool jobs, a working Voiceflow assistant, and a documented need for Make scenarios connecting JobTread API and Airtable memory so the assistant can answer job-state questions and later take actions</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>Voiceflow-JobTread-Airtable phase-1 build</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L52" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>Manual follow-up only; lead with read-only JobTread sync plus Airtable memory before write actions</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O52" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P52" t="str">
+        <x:v>Clear buyer pain, detailed scope, and natural fixed-scope first milestone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>C10K-051</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Cafe Manager / Toast POS reporting fix</x:v>
+      </x:c>
+      <x:c r="E53"/>
+      <x:c r="F53" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>https://community.make.com/t/toast-pos-make-google-sheets-help/108218</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>Dashboard/reporting cleanup</x:v>
+      </x:c>
+      <x:c r="I53" t="str">
+        <x:v>Restaurant operator says Toast API data already lands in Make and Google Sheets but totals do not match Toast Sales Summary because aggregation lives in Sheets and duplicate or partial runs corrupt reporting</x:v>
+      </x:c>
+      <x:c r="J53" t="str">
+        <x:v>Idempotent POS reporting reconciliation sprint</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L53" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M53" t="str">
+        <x:v>Manual follow-up only; lead with moving aggregation and dedupe into Make and defining a reconciled summary table</x:v>
+      </x:c>
+      <x:c r="N53" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O53" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P53" t="str">
+        <x:v>Strong short-cycle debug-and-finish opportunity with exact acceptance criterion: totals must match Toast daily summary</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>C10K-052</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>StartAI</x:v>
+      </x:c>
+      <x:c r="E54"/>
+      <x:c r="F54" t="str">
+        <x:v>Wellfound public listing</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>https://wellfound.com/jobs/3533470-airtable-specialist-automations-configuration</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>Airtable CRM/dashboard automation</x:v>
+      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>Wellfound listing posted May 8, 2026 describes a freelance or part-time Airtable specialist role for building bases, automations, dashboards, and integrations with Slack, Google Workspace, Stripe, and CRMs for digital businesses and agencies</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>Airtable automation and CRM systems sprint</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L54" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>Manual follow-up only; if pursued, frame as project-based Airtable cleanup plus automation package rather than open-ended staffing</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O54" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P54" t="str">
+        <x:v>Fresh listing with recruiter active and project-based option explicitly allowed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>C10K-053</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>MVM Management Company</x:v>
+      </x:c>
+      <x:c r="E55"/>
+      <x:c r="F55" t="str">
+        <x:v>Wellfound public listing</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>https://wellfound.com/jobs/3844627-airtable-architect-automation-specialist</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>Internal tools / Airtable stabilization</x:v>
+      </x:c>
+      <x:c r="I55" t="str">
+        <x:v>Wellfound listing posted May 8, 2026 describes a contract part-time Airtable Architect &amp; Automation Specialist to design, stabilize, and automate internal operational systems across multiple teams with Airtable, Zapier, and Make</x:v>
+      </x:c>
+      <x:c r="J55" t="str">
+        <x:v>Airtable stabilization and internal-ops refactor sprint</x:v>
+      </x:c>
+      <x:c r="K55" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L55" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M55" t="str">
+        <x:v>Manual follow-up only; best angle is audit-plus-refactor for existing Airtable systems with reliability and role-based views</x:v>
+      </x:c>
+      <x:c r="N55" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O55" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P55" t="str">
+        <x:v>Higher-quality contract signal than generic hiring posts because the pain is existing-system stability and error reduction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>C10K-054</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>Archestra</x:v>
+      </x:c>
+      <x:c r="E56"/>
+      <x:c r="F56" t="str">
+        <x:v>Algora public bounty page</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>https://algora.io/archestra-ai</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>AI workflow infrastructure bounty</x:v>
+      </x:c>
+      <x:c r="I56" t="str">
+        <x:v>Algora shows open bounties as of this run including a USD 1500 Unified OpenAI-format LLM proxy endpoint and smaller queue, budgeting, and MCP admin tasks for an enterprise MCP gateway and orchestrator</x:v>
+      </x:c>
+      <x:c r="J56" t="str">
+        <x:v>Targeted bounty implementation</x:v>
+      </x:c>
+      <x:c r="K56" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L56" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M56" t="str">
+        <x:v>Review issue scope before any build commitment; prioritize the USD 1500 proxy endpoint only if the spec is narrow enough for a bounded delivery</x:v>
+      </x:c>
+      <x:c r="N56" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O56" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P56" t="str">
+        <x:v>Not buyer outreach; included because it is a live public bounty source directly relevant to AI workflow infrastructure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>C10K-055</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>Claire Manwaring / caregiver SMS app</x:v>
+      </x:c>
+      <x:c r="E57"/>
+      <x:c r="F57" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>https://community.make.com/t/looking-for-short-term-help-with-make-bubble-supabase-claude-twilio/108581</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>AI workflow automation / lead-intake-style messaging</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>Make Community post from May 7, 2026 seeks a short-term freelancer for a mid-May build using Bubble, Supabase, Make, Twilio, Claude, Slack review, and analytics to run stateful SMS caregiver flows</x:v>
+      </x:c>
+      <x:c r="J57" t="str">
+        <x:v>Stateful SMS and HITL workflow sprint</x:v>
+      </x:c>
+      <x:c r="K57" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L57" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M57" t="str">
+        <x:v>Manual follow-up only; lead with a bounded 3-4 week state machine plus human-review build, not open-ended staffing</x:v>
+      </x:c>
+      <x:c r="N57" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O57" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P57" t="str">
+        <x:v>Strong because it names the stack the buyer already chose and the build window is immediate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>C10K-056</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>Nikolaos Zissidis / e-commerce brand</x:v>
+      </x:c>
+      <x:c r="E58"/>
+      <x:c r="F58" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>https://community.n8n.io/t/hiring-n8n-automation-specialist-paid-long-term-remote-e-commerce-shopify/284836</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>Content workflow automation</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>n8n Community post from April 5, 2026 asks for a paid n8n workflow that turns competitor scripts into short-form videos using Google Drive, Claude API, and AI video tooling for 10+ social accounts</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>AI video content pipeline v1</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L58" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>Manual follow-up only; best angle is a bounded content-pipeline v1 with approval checkpoints and export handoff</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O58" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P58" t="str">
+        <x:v>Project is concrete enough for a fixed-scope first release even though the thread mentions long-term potential</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>C10K-057</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>GeniusAISolutions</x:v>
+      </x:c>
+      <x:c r="E59"/>
+      <x:c r="F59" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>https://community.n8n.io/t/looking-for-n8n-expert-for-paid-debugging-session-whatsapp-airtable-openai-workflow/276670</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>CRM / messaging workflow debugging</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>n8n Community post from March 13, 2026 asks for a paid 1-2 hour debugging session on a WhatsApp Cloud API, Airtable state machine, OpenAI, and Telegram handoff workflow with bugs in state logic and escalation</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>Paid workflow audit and fix plan</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>Manual follow-up only; angle should be a paid race-condition and handoff-state audit with a short remediation plan</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="O59" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P59" t="str">
+        <x:v>Very small entry offer and explicit budget openness make this a clean consult-sized opportunity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>C10K-058</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>Christian Tekwe / ProductBuilder SaaS</x:v>
+      </x:c>
+      <x:c r="E60"/>
+      <x:c r="F60" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>https://community.make.com/t/hiring-make-com-specialist-for-multi-client-content-automation-saas-ai-apis-airtable-publishing-workflows/103804</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>AI publishing workflow automation</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>Make Community post from February 18, 2026 describes a 3-module pipeline using Claude API, Airtable, and automated publishing for 20+ creator clients in a health and wellness content SaaS</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Research-and-scoring module sprint</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>monitor_only_qualified</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>Manual follow-up only; propose module 1 research-and-scoring first, then expand if reliability is proven</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="O60" t="str">
+        <x:v>docs/opportunity-log.md</x:v>
+      </x:c>
+      <x:c r="P60" t="str">
+        <x:v>Good fit because the buyer already decomposed the system into modules and multi-client parameterization is explicit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>C10K-059</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>2026-05-09</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>Synergy Effect / Tomas Maciulskas</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>info@s-e.lt</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>n8n Community public post</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>https://community.n8n.io/t/hiring-ai-automation-engineer-n8n-ai-agent-developer/294904</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>AI automation / n8n project delivery</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>Fresh May 7 2026 post asks for project-based freelance/contractor cooperation building production-ready n8n, AI agent, RPA, OCR, CRM/ERP, finance/logistics/customer-support and HITL automations</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>Project-based AI automation delivery packet</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>Watch for reply; if positive, request one real process, systems involved, target output, sample records, and quote a USD 1800-4500 fixed milestone</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O61" t="str">
+        <x:v>gmail:19e0fb48b5c32d18; synergy-effect-ai-automation.html; docs/synergy-effect-ai-automation-proposal.md; scripts/check-email-cadence.mjs</x:v>
+      </x:c>
+      <x:c r="P61" t="str">
+        <x:v>Sent fixed-scope project-delivery response to info@s-e.lt after May 10 cadence gate allowed; positioned as project-based independent freelancer, not employee role, with public technical packet and sample workflow links.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Send SoIN launch QA proposal
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re6f9886675974a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R23de9e3f5dcc4066"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R707dd836e63a4c33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rf97b20dba48b4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R02afd8b8b9f749a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rb055699a8756408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rdb2c7682147f42cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R9c1a223c81d0477d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2823,20 +2823,22 @@
         <x:v>CMS/CRM/partner portal launch QA support</x:v>
       </x:c>
       <x:c r="K49" t="str">
-        <x:v>proposal_packet_ready_no_gmail</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L49" t="str">
-        <x:v>2026-05-09</x:v>
+        <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M49" t="str">
-        <x:v>Use non-Gmail RFP submission route or manual-approved channel; do not send via Gmail unless user reverses instruction</x:v>
-      </x:c>
-      <x:c r="N49"/>
+        <x:v>Watch for reply; if positive, request staging/vendor-selection window and convert USD 8500 support slice into final one-page scope, acceptance criteria, and payment link/invoice</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
       <x:c r="O49" t="str">
-        <x:v>docs/outbox-next.md</x:v>
+        <x:v>gmail:19e0fd37e18291d8; outputs/codex10k/soin_launch_qa_support_proposal.pdf; docs/outbox-next.md</x:v>
       </x:c>
       <x:c r="P49" t="str">
-        <x:v>Preparing USD 8500 bounded launch-QA support proposal; no individual pre-submission meeting request; no visitor/partner/CRM production data by email</x:v>
+        <x:v>Sent USD 8500 bounded launch-QA support option with verified PDF attachment. No individual pre-submission meeting request; no visitor, partner, or CRM production data by email.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">

</xml_diff>

<commit_message>
Add 3D Walkabout outreach packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R02afd8b8b9f749a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rb055699a8756408f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rdb2c7682147f42cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R9c1a223c81d0477d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3238029187ea45dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rbcdd8aadee644d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rf3b15024f1f94c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Re04ccac0fd7e41b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3545,22 +3545,22 @@
         <x:v>Lead-gen proof-of-concept pipeline</x:v>
       </x:c>
       <x:c r="K64" t="str">
-        <x:v>monitor_only_qualified</x:v>
+        <x:v>packet_prepared_for_forum_dm</x:v>
       </x:c>
       <x:c r="L64" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M64" t="str">
-        <x:v>Manual follow-up only; best angle is one proof-of-concept source and scoring pipeline before a larger retained build</x:v>
+        <x:v>Use forum DM/reply only if platform access is available; do not email third-party responder addresses; if positive, request approved source, ICP, allowed enrichment fields, and output schema</x:v>
       </x:c>
       <x:c r="N64" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O64" t="str">
-        <x:v>docs/opportunity-log.md</x:v>
+        <x:v>docs/opportunity-log.md; darius-leadgen-poc.html</x:v>
       </x:c>
       <x:c r="P64" t="str">
-        <x:v>High buyer intent because the requester wants architecture guidance and proof with real data before full payment</x:v>
+        <x:v>Prepared compliance-bounded source-to-review POC page; public email in thread belonged to another respondent, not the buyer</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3849,6 +3849,56 @@
       </x:c>
       <x:c r="P70" t="str">
         <x:v>Small GitHub-style paid workflow opportunity rather than outreach lead</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>C10K-069</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>3D Walkabout / Tim Brickle</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>tim@3dwalkabout.com.au</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Make Community public post / official company contact</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>https://community.make.com/t/need-a-pro-to-help-with-hubspot-clickup-intergration/107582</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>CRM / task automation</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>April 17, 2026 Make Community post asks for an experienced Make specialist to build and stabilize HubSpot-to-ClickUp automations including deal-stage triggers, writebacks, duplicate prevention, correct filtering, and simplifying messy scenarios</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>HubSpot-ClickUp reliability sprint</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>packet_prepared_pending_send</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>Send fixed-scope USD 1800 reliability-sprint email after cadence gate and public page publish; if positive, request current scenario, trigger stages, target ClickUp list, and sample deals</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O71" t="str">
+        <x:v>3dwalkabout-hubspot-clickup.html; https://3dwalkabout.com.au/contact/; public company email evidence</x:v>
+      </x:c>
+      <x:c r="P71" t="str">
+        <x:v>Direct public buyer pain with official contact and company site; constrain data handling to least-privilege or sample records because CRM data can contain customer/deal info</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record 3D Walkabout outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3238029187ea45dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rbcdd8aadee644d74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rf3b15024f1f94c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Re04ccac0fd7e41b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd69f617161ee4a00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Raa75a9e569ec4643"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rbfa6888fde6b4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbe3dba54eb6140cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3883,22 +3883,22 @@
         <x:v>HubSpot-ClickUp reliability sprint</x:v>
       </x:c>
       <x:c r="K71" t="str">
-        <x:v>packet_prepared_pending_send</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L71" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M71" t="str">
-        <x:v>Send fixed-scope USD 1800 reliability-sprint email after cadence gate and public page publish; if positive, request current scenario, trigger stages, target ClickUp list, and sample deals</x:v>
+        <x:v>Watch for reply; if positive, request current scenario, trigger stages, target ClickUp list, sample deals, and quote USD 1800 reliability sprint acceptance checklist</x:v>
       </x:c>
       <x:c r="N71" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O71" t="str">
-        <x:v>3dwalkabout-hubspot-clickup.html; https://3dwalkabout.com.au/contact/; public company email evidence</x:v>
+        <x:v>gmail:19e0feb8882b174a; 3dwalkabout-hubspot-clickup.html; https://3dwalkabout.com.au/contact/; public company email evidence</x:v>
       </x:c>
       <x:c r="P71" t="str">
-        <x:v>Direct public buyer pain with official contact and company site; constrain data handling to least-privilege or sample records because CRM data can contain customer/deal info</x:v>
+        <x:v>Sent fixed-scope USD 1800 HubSpot-ClickUp reliability sprint after live packet URL returned 200; constrain data handling to least-privilege or sample records because CRM data can contain customer/deal info</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Prepare SnipeAgent SMS automation packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd69f617161ee4a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Raa75a9e569ec4643"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rbfa6888fde6b4d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbe3dba54eb6140cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcdad83b42a2841df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rc606924b3cce4d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rd505464e4a3b409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rf968d531c6424a5b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3901,6 +3901,106 @@
         <x:v>Sent fixed-scope USD 1800 HubSpot-ClickUp reliability sprint after live packet URL returned 200; constrain data handling to least-privilege or sample records because CRM data can contain customer/deal info</x:v>
       </x:c>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>C10K-070</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>SnipeAgent / Alex T</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>contact@snipeagent.ai</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Make Community public post</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>https://community.make.com/t/make-com-expert-needed-ai-powered-sms-automation-system-full-build/106574</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>SMS / MMS AI automation</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>March 27, 2026 Make Community post asks for a fixed-price AI-powered SMS automation system with 6 scenarios, about 41 modules, Sinch SMS/MMS, Claude Haiku, Rainforest API, SerpApi, Carrd webhook, parallel API calls, MMS image handling, E.164 normalization, per-user processing locks, data stores, and re-engagement sequences</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>SMS automation architecture pass and build</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>packet_prepared_pending_send</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>Send after cadence gate and public page publish; if positive, request NDA/full scope, test number/webhook path, API access rules, reply format, and milestone demo expectations</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O72" t="str">
+        <x:v>snipeagent-sms-automation.html; assets/snipeagent-sms-workflow-visual.png; https://community.make.com/t/make-com-expert-needed-ai-powered-sms-automation-system-full-build/106574</x:v>
+      </x:c>
+      <x:c r="P72" t="str">
+        <x:v>Direct buyer email listed in the post; frame as USD 400 architecture pass credited toward USD 2400 build; no unsolicited SMS or production phone data by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>C10K-071</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Ferncliff Camp and Conference Center</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>info@ferncliff.org</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>Official RFP page</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>https://ferncliff.org/about/jobs/rfps/</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>Website / CMS launch QA</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>May 2026 public RFP seeks website redesign and CMS support with user pathways, mobile-first design, accessibility expectations, and handoffs to CampBrain, DonorPerfect, Constant Contact, ADP, and Square; proposals due May 25, 2026</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>Website launch QA and CMS handoff support</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>packet_prepared_monitor</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>Use official RFP submission/contact path only; if pursuing, frame as independent USD 3800 launch-QA sidecar for selected vendor or internal team, not a prime redesign bid</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>2026-05-15</x:v>
+      </x:c>
+      <x:c r="O73" t="str">
+        <x:v>ferncliff-launch-qa-support.html; https://ferncliff.org/about/jobs/rfps/</x:v>
+      </x:c>
+      <x:c r="P73" t="str">
+        <x:v>Prepared public-safe support page; verify current RFP email/instructions before any outreach</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Record SnipeAgent outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcdad83b42a2841df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rc606924b3cce4d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rd505464e4a3b409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rf968d531c6424a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbe3cedab9ab348b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rf92fa5972d954460"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2ee6204288db4d00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R22fa12f617a74c8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3933,22 +3933,22 @@
         <x:v>SMS automation architecture pass and build</x:v>
       </x:c>
       <x:c r="K72" t="str">
-        <x:v>packet_prepared_pending_send</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L72" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M72" t="str">
-        <x:v>Send after cadence gate and public page publish; if positive, request NDA/full scope, test number/webhook path, API access rules, reply format, and milestone demo expectations</x:v>
+        <x:v>Watch for reply; if positive, request NDA/full scope, test number/webhook path, API access rules, reply format, milestone demo expectations, and convert USD 400 architecture pass into payment request</x:v>
       </x:c>
       <x:c r="N72" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O72" t="str">
-        <x:v>snipeagent-sms-automation.html; assets/snipeagent-sms-workflow-visual.png; https://community.make.com/t/make-com-expert-needed-ai-powered-sms-automation-system-full-build/106574</x:v>
+        <x:v>gmail:19e0ffab0e946f49; snipeagent-sms-automation.html; assets/snipeagent-sms-workflow-visual.png; https://community.make.com/t/make-com-expert-needed-ai-powered-sms-automation-system-full-build/106574</x:v>
       </x:c>
       <x:c r="P72" t="str">
-        <x:v>Direct buyer email listed in the post; frame as USD 400 architecture pass credited toward USD 2400 build; no unsolicited SMS or production phone data by email</x:v>
+        <x:v>Sent USD 400 architecture pass credited toward USD 2400 build after live packet returned 200; direct buyer email listed in the post; no unsolicited SMS or production phone data by email</x:v>
       </x:c>
     </x:row>
     <x:row r="73">

</xml_diff>

<commit_message>
Prepare Chek Creative partner pilot
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbe3cedab9ab348b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rf92fa5972d954460"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2ee6204288db4d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R22fa12f617a74c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5727011b130d4de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Raf55c7eb963841c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rc891d8f1bb3c4b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R8e0ec735a0394138"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4001,6 +4001,56 @@
         <x:v>Prepared public-safe support page; verify current RFP email/instructions before any outreach</x:v>
       </x:c>
     </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>C10K-072</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>Chek Creative / Josh</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>hello@chekcreative.com</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Make Community public post / official contact page</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>https://community.make.com/t/hiring-senior-make-com-automation-engineers-ongoing-contractor-work-75-95-hr/105775</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Agency automation partner work</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>March 17, 2026 Make Community post says Chek Creative is building a senior Make.com automation bench for CRM, marketing ops, lead attribution, APIs, webhooks, CMS-related work, error handling, retries, logging, idempotency, and async-first client communication; official site lists hello@chekcreative.com</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>Automation partner pilot</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>packet_prepared_pending_send</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>Send after cadence gate and live page publish; if positive, request one client-safe workflow brief, tools involved, source-of-truth app, sample payloads, and documentation preference</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>chek-automation-partner-pilot.html; https://www.chekcreative.com/contact/; https://community.make.com/t/hiring-senior-make-com-automation-engineers-ongoing-contractor-work-75-95-hr/105775</x:v>
+      </x:c>
+      <x:c r="P74" t="str">
+        <x:v>Frame as USD 1200 paid pilot rather than job application; no client secrets or private workflows by email</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Record Chek Creative outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5727011b130d4de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Raf55c7eb963841c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rc891d8f1bb3c4b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R8e0ec735a0394138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4f2e0f7280204ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Reaa0bb4e197e40e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R807e7a73315f4584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rcbb637297a224f97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4033,22 +4033,22 @@
         <x:v>Automation partner pilot</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>packet_prepared_pending_send</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L74" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M74" t="str">
-        <x:v>Send after cadence gate and live page publish; if positive, request one client-safe workflow brief, tools involved, source-of-truth app, sample payloads, and documentation preference</x:v>
+        <x:v>Watch for reply; if positive, request one client-safe workflow brief, tools involved, source-of-truth app, sample payloads, documentation preference, and convert USD 1200 pilot into payment request</x:v>
       </x:c>
       <x:c r="N74" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O74" t="str">
-        <x:v>chek-automation-partner-pilot.html; https://www.chekcreative.com/contact/; https://community.make.com/t/hiring-senior-make-com-automation-engineers-ongoing-contractor-work-75-95-hr/105775</x:v>
+        <x:v>gmail:19e10093fb4ce954; chek-automation-partner-pilot.html; https://www.chekcreative.com/contact/; https://community.make.com/t/hiring-senior-make-com-automation-engineers-ongoing-contractor-work-75-95-hr/105775</x:v>
       </x:c>
       <x:c r="P74" t="str">
-        <x:v>Frame as USD 1200 paid pilot rather than job application; no client secrets or private workflows by email</x:v>
+        <x:v>Sent USD 1200 paid pilot after live packet returned 200; framed as paid pilot rather than job application; no client secrets or private workflows by email</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Prepare NVTA ADA QA quote
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4f2e0f7280204ee1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Reaa0bb4e197e40e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R807e7a73315f4584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rcbb637297a224f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd4c3e86a8d814805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rd4cac002a76e41c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rf4f46b70e9be4982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R69f1a9db0fd54c47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3983,22 +3983,22 @@
         <x:v>Website launch QA and CMS handoff support</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>packet_prepared_monitor</x:v>
+        <x:v>duplicate_packet_do_not_send</x:v>
       </x:c>
       <x:c r="L73" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M73" t="str">
-        <x:v>Use official RFP submission/contact path only; if pursuing, frame as independent USD 3800 launch-QA sidecar for selected vendor or internal team, not a prime redesign bid</x:v>
+        <x:v>Do not send as a new outreach because Ferncliff was already contacted as C10K-039; use this page only if Ferncliff replies or asks for an updated support packet</x:v>
       </x:c>
       <x:c r="N73" t="str">
         <x:v>2026-05-15</x:v>
       </x:c>
       <x:c r="O73" t="str">
-        <x:v>ferncliff-launch-qa-support.html; https://ferncliff.org/about/jobs/rfps/</x:v>
+        <x:v>ferncliff-launch-qa-support.html; data/prospects.csv:C10K-039; https://ferncliff.org/about/jobs/rfps/</x:v>
       </x:c>
       <x:c r="P73" t="str">
-        <x:v>Prepared public-safe support page; verify current RFP email/instructions before any outreach</x:v>
+        <x:v>Prepared public-safe support page, but dedupe found prior C10K-039 Gmail outreach to Kimberly/info; avoid duplicate procurement contact</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -4049,6 +4049,56 @@
       </x:c>
       <x:c r="P74" t="str">
         <x:v>Sent USD 1200 paid pilot after live packet returned 200; framed as paid pilot rather than job application; no client secrets or private workflows by email</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>C10K-073</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Napa Valley Transportation Authority</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>procurements@nvta.ca.gov; rcoombs@nvta.ca.gov</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>Official RFQ page / RFQ PDF</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>https://nvta.ca.gov/procurements/rfq-26-r08-for-ada-website-compliance/</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>Website accessibility QA</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>Official RFQ 26-R08 requests ADA website compliance support for NVTA.ca.gov and VineTransit.com against WCAG 2.2 AA; quotes due May 22, 2026 at 2:00 PM local time and inquiries/submissions go to procurements@nvta.ca.gov copy rcoombs@nvta.ca.gov</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>ADA website QA sidecar quote</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>packet_prepared_pending_send</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>Send after cadence gate and live page publish with PDF attachment; if positive, request priority URLs, representative PDFs/documents, preferred tracker format, remediation owner, and procurement/payment path</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O75" t="str">
+        <x:v>nvta-ada-qa-sidecar.html; assets/nvta-ada-qa-visual.png; outputs/codex10k/nvta_ada_qa_sidecar_quote.pdf; https://nvta.ca.gov/wp-content/uploads/2026/04/RFQ-26-R08-ADA-Website-ComplianceFD.pdf</x:v>
+      </x:c>
+      <x:c r="P75" t="str">
+        <x:v>Frame as limited USD 4800 QA/retest/staff-checklist sidecar, not legal certification or full remediation/maintenance prime</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record NVTA quote send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rd4c3e86a8d814805"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rd4cac002a76e41c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rf4f46b70e9be4982"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R69f1a9db0fd54c47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0dd543ffde2a4f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R869032a0c7d843ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R1d995ddf1fe24449"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rd7e3fae26c934822"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4083,22 +4083,22 @@
         <x:v>ADA website QA sidecar quote</x:v>
       </x:c>
       <x:c r="K75" t="str">
-        <x:v>packet_prepared_pending_send</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L75" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M75" t="str">
-        <x:v>Send after cadence gate and live page publish with PDF attachment; if positive, request priority URLs, representative PDFs/documents, preferred tracker format, remediation owner, and procurement/payment path</x:v>
+        <x:v>Watch for procurement response; if positive, request priority URLs, representative PDFs/documents, preferred tracker format, remediation owner, and procurement/payment path</x:v>
       </x:c>
       <x:c r="N75" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O75" t="str">
-        <x:v>nvta-ada-qa-sidecar.html; assets/nvta-ada-qa-visual.png; outputs/codex10k/nvta_ada_qa_sidecar_quote.pdf; https://nvta.ca.gov/wp-content/uploads/2026/04/RFQ-26-R08-ADA-Website-ComplianceFD.pdf</x:v>
+        <x:v>gmail:19e101890b095ee2; nvta-ada-qa-sidecar.html; assets/nvta-ada-qa-visual.png; outputs/codex10k/nvta_ada_qa_sidecar_quote.pdf; https://nvta.ca.gov/wp-content/uploads/2026/04/RFQ-26-R08-ADA-Website-ComplianceFD.pdf</x:v>
       </x:c>
       <x:c r="P75" t="str">
-        <x:v>Frame as limited USD 4800 QA/retest/staff-checklist sidecar, not legal certification or full remediation/maintenance prime</x:v>
+        <x:v>Sent formal RFQ 26-R08 quote with USD 4800 limited QA/retest/staff-checklist sidecar and PDF attachment after live page returned 200; not legal certification or full remediation/maintenance prime</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record Duck proposal send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0dd543ffde2a4f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R869032a0c7d843ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R1d995ddf1fe24449"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rd7e3fae26c934822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1e46f19bf04d4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rdb5c0681977a4988"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2016e0cf612c4566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R70e9fea705454666"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4101,6 +4101,56 @@
         <x:v>Sent formal RFQ 26-R08 quote with USD 4800 limited QA/retest/staff-checklist sidecar and PDF attachment after live page returned 200; not legal certification or full remediation/maintenance prime</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>C10K-074</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Town of Duck NC</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>knickens@ducknc.gov</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Official RFP page / RFP PDF</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>https://ducknc.gov/news/request-for-proposals-website-redesign-cms-implementation/</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>Municipal website launch QA</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>Official Town of Duck RFP issued April 23 2026 requests website redesign and CMS implementation with ADA, Section 508, WCAG 2.2 AA, automated scanning/reporting, content migration, searchable documents, analytics, staff training, security, hosting, and post-launch support; proposals due May 14 2026 at 5:00 PM EST and electronic submissions are acceptable</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>Launch-QA accessibility and CMS handoff sidecar</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>Watch for procurement response; if positive, request priority pages, representative PDFs/forms/events, staging access timing, preferred tracker format, remediation owner, and procurement/payment path</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O76" t="str">
+        <x:v>gmail:19e10294ab3b5ab5; duck-ada-launch-qa-sidecar.html; outputs/codex10k/town_of_duck_launch_qa_sidecar_proposal.pdf; https://ducknc.gov/wp-content/uploads/2026/04/Town-of-Duck-Website-RFP-2026-04-23.pdf</x:v>
+      </x:c>
+      <x:c r="P76" t="str">
+        <x:v>Sent USD 6800 limited launch-QA/accessibility/CMS handoff sidecar with PDF attachment after public page returned 200; not a full redesign bid, legal certification, hosting proposal, CMS license, or long-term maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Prepare Ely migration QA proposal
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1e46f19bf04d4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rdb5c0681977a4988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2016e0cf612c4566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R70e9fea705454666"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5df7d0f340e34caa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R6f70e7227a3f41d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R60658ce5f8a84b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R9f63a0c648c9448d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4151,6 +4151,56 @@
         <x:v>Sent USD 6800 limited launch-QA/accessibility/CMS handoff sidecar with PDF attachment after public page returned 200; not a full redesign bid, legal certification, hosting proposal, CMS license, or long-term maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>C10K-075</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Ely Area Tourism Bureau / Ely Chamber of Commerce</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>jess@rootbeerlady.com</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Official RFP page / RFP PDF</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>https://www.ely.org/rfp/</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>Tourism CMS migration QA</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>Official Ely RFP requests website redesign and content migration from Simpleview with 50-70 pages, business/member directory data, listings, forms, online shop, SEO preservation, analytics, WCAG 2.1 AA accessibility, CMS training, QA, launch support, and 90-day post-launch support; proposals due May 11 2026</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>Migration QA directory readiness and launch support slice</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>prepared_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>Run cadence gate after 2026-05-10T04:48:31Z; if allowed, send formal limited USD 12500 sidecar proposal PDF and public page link</x:v>
+      </x:c>
+      <x:c r="N77" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O77" t="str">
+        <x:v>ely-migration-qa-sidecar.html; outputs/codex10k/ely_migration_qa_launch_readiness_proposal.pdf; https://assets.simpleviewinc.com/simpleview/image/upload/v1/clients/elymn/Request_for_Proposal_Website_Development_Content_Migration_2__3348aec4-e026-4d13-84d5-183b749bb1ab.pdf</x:v>
+      </x:c>
+      <x:c r="P77" t="str">
+        <x:v>Prepared non-n8n tourism CMS migration QA packet; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or ongoing maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Record Ely proposal send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5df7d0f340e34caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R6f70e7227a3f41d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R60658ce5f8a84b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R9f63a0c648c9448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rad34107b28674e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4d5b7d1b3fed4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R0f1182c237e04d50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbbeaed48741b4cf9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4183,22 +4183,22 @@
         <x:v>Migration QA directory readiness and launch support slice</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>prepared_fixed_scope</x:v>
+        <x:v>contacted_fixed_scope</x:v>
       </x:c>
       <x:c r="L77" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M77" t="str">
-        <x:v>Run cadence gate after 2026-05-10T04:48:31Z; if allowed, send formal limited USD 12500 sidecar proposal PDF and public page link</x:v>
+        <x:v>Watch for RFP response; if positive, request current crawl/export, representative listing export, staging/vendor timeline, preferred tracker format, and procurement/payment path</x:v>
       </x:c>
       <x:c r="N77" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O77" t="str">
-        <x:v>ely-migration-qa-sidecar.html; outputs/codex10k/ely_migration_qa_launch_readiness_proposal.pdf; https://assets.simpleviewinc.com/simpleview/image/upload/v1/clients/elymn/Request_for_Proposal_Website_Development_Content_Migration_2__3348aec4-e026-4d13-84d5-183b749bb1ab.pdf</x:v>
+        <x:v>gmail:19e1037e9f166d0a; ely-migration-qa-sidecar.html; outputs/codex10k/ely_migration_qa_launch_readiness_proposal.pdf; https://assets.simpleviewinc.com/simpleview/image/upload/v1/clients/elymn/Request_for_Proposal_Website_Development_Content_Migration_2__3348aec4-e026-4d13-84d5-183b749bb1ab.pdf</x:v>
       </x:c>
       <x:c r="P77" t="str">
-        <x:v>Prepared non-n8n tourism CMS migration QA packet; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or ongoing maintenance contract</x:v>
+        <x:v>Sent USD 12500 limited migration-QA/directory-readiness/launch-support sidecar with PDF attachment after public page returned 200; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or ongoing maintenance contract</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Track non-n8n portal opportunities
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rad34107b28674e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4d5b7d1b3fed4cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R0f1182c237e04d50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbbeaed48741b4cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd5cd0e5d558420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Ra502c9cf2f884f84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Red78288714ad4020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R666a030551d240e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4201,6 +4201,154 @@
         <x:v>Sent USD 12500 limited migration-QA/directory-readiness/launch-support sidecar with PDF attachment after public page returned 200; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or ongoing maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>C10K-076</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Superior Court of California County of Placer</x:v>
+      </x:c>
+      <x:c r="E78"/>
+      <x:c r="F78" t="str">
+        <x:v>Bonfire portal / public procurement mirror</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>https://lacourt.bonfirehub.com/opportunities/233058</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>Power BI dashboard modernization</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>Public procurement mirror for SP-2026-0010 says Placer Court seeks Power BI development services to update rebuild and modernize about 20 existing dashboards across court operational data including eCourt Tyler jury and internal sources; responses due May 13 2026 through Bonfire</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>Power BI dashboard modernization QA/UAT support</x:v>
+      </x:c>
+      <x:c r="K78" t="str">
+        <x:v>monitor_portal_qualified</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M78" t="str">
+        <x:v>Portal-only path; prepare only if Bonfire account/access is available or if a prime/subcontractor path appears; do not email unsolicited</x:v>
+      </x:c>
+      <x:c r="N78" t="str">
+        <x:v>2026-05-12</x:v>
+      </x:c>
+      <x:c r="O78" t="str">
+        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/sp-2026-0010-power-bi-development-services-for-placer-court-sp20260010</x:v>
+      </x:c>
+      <x:c r="P78" t="str">
+        <x:v>Non-n8n analytics/data lane; likely requires formal portal response, insurance, business licensing, and procurement forms; best as portal-ready packet or subcontracted QA/UAT workstream</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>C10K-077</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Railroad Commission of Texas</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>reese.miller@rrc.texas.gov</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>TxSmartBuy ESBD / RRC solicitations</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>https://www.txsmartbuy.gov/esbd/455-26-1018</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>Salesforce implementation QA</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>Public sources for RFO 455-26-1018 say RRC seeks Salesforce and tools implementation services and support across Salesforce platform modernization and related tools; responses due May 19 2026 via Texas procurement channels</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>Salesforce implementation QA and requirements traceability sidecar</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>monitor_portal_qualified</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>Portal/procurement path; do not send as casual outreach; if pursuing, prepare subcontractor/QA packet around requirements traceability, migration QA, UAT scripts, dashboard acceptance, and defect triage</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O79" t="str">
+        <x:v>https://www.rrc.texas.gov/about-us/contract-management/solicitations/; https://www.txsmartbuy.gov/esbd/455-26-1018</x:v>
+      </x:c>
+      <x:c r="P79" t="str">
+        <x:v>Non-n8n Salesforce/data migration lane; likely requires Texas procurement compliance and prime/vendor credentials; better as named QA specialist or subcontract support</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>C10K-078</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Missouri Office of State Public Defender</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>procurement@mspd.mo.gov</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>MissouriBUYS / public procurement mirror</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>https://missouribuys.mo.gov</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Case-management migration QA</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>Public sources for MSPD 0000000003SL say Missouri State Public Defender seeks an integrated public defense management system covering case management, portals, court integrations, workflow automation, analytics, HCL Notes/Domino migration, and statewide rollout; proposals due June 30 2026 via MissouriBUYS</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>Migration and implementation QA sidecar</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>monitor_portal_qualified</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>Portal/procurement path with large prime scope; prepare only as subcontractor/QA sidecar unless full vendor team appears</x:v>
+      </x:c>
+      <x:c r="N80" t="str">
+        <x:v>2026-05-20</x:v>
+      </x:c>
+      <x:c r="O80" t="str">
+        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/request-for-proposal-rfp-for-an-integrated-public-defense-management-system-300000235023766</x:v>
+      </x:c>
+      <x:c r="P80" t="str">
+        <x:v>Non-n8n public-sector migration lane; strong fit for migration risk register, sample data validation, UAT/go-live templates, weekly status/reporting pack; too large for solo prime</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Record Hiawatha proposal send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rfd5cd0e5d558420d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Ra502c9cf2f884f84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Red78288714ad4020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R666a030551d240e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re4d4ace5435c4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R5a1a4bff739a4645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2ac34bbb10444a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rd6b2c683848b4cee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4349,6 +4349,56 @@
         <x:v>Non-n8n public-sector migration lane; strong fit for migration risk register, sample data validation, UAT/go-live templates, weekly status/reporting pack; too large for solo prime</x:v>
       </x:c>
     </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>C10K-079</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Hiawatha Academies</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>kgroves@hiawathaacademies.org</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Official RFQ page / RFQ PDF</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>https://www.hiawathaacademies.org/apps/pages/index.jsp?uREC_ID=2019187&amp;type=d&amp;pREC_ID=2642881</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>School website multilingual accessibility QA</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>Official RFQ issued April 15 2026 requests website redesign development hosting and implementation for a charter school network serving about 1600 students, with WCAG 2.1 A/AA, mobile responsiveness, English/Spanish/Somali support, content migration, recruitment, family engagement, and communications; proposals due May 15 2026 at 11:59 PM</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>Multilingual/accessibility/content-migration launch QA sidecar</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>Watch for RFQ response/confirmation; if positive, request staging/vendor timeline, representative URLs/templates, language sample paths, preferred tracker format, and procurement/payment path</x:v>
+      </x:c>
+      <x:c r="N81" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O81" t="str">
+        <x:v>gmail:19e104c1b35de655; hiawatha-school-website-qa-sidecar.html; outputs/codex10k/hiawatha_school_website_qa_sidecar_proposal.pdf; https://www.hiawathaacademies.org/apps/pages/index.jsp?uREC_ID=2019187&amp;type=d&amp;pREC_ID=2642881</x:v>
+      </x:c>
+      <x:c r="P81" t="str">
+        <x:v>Sent USD 12000 limited multilingual/accessibility/content-migration QA sidecar with PDF attachment after cadence gate returned allowed and public page/PDF returned 200; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or long-term maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Prepare Placer Power BI portal packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Re4d4ace5435c4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R5a1a4bff739a4645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R2ac34bbb10444a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rd6b2c683848b4cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rba9cd545e0ff48fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Ra10f7261f1704caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R33cf8727c82042aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0d1bbacf399e436a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4219,34 +4219,34 @@
         <x:v>Bonfire portal / public procurement mirror</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>https://lacourt.bonfirehub.com/opportunities/233058</x:v>
+        <x:v>https://lacourt.bonfirehub.com/portal/?tab=openOpportunities</x:v>
       </x:c>
       <x:c r="H78" t="str">
         <x:v>Power BI dashboard modernization</x:v>
       </x:c>
       <x:c r="I78" t="str">
-        <x:v>Public procurement mirror for SP-2026-0010 says Placer Court seeks Power BI development services to update rebuild and modernize about 20 existing dashboards across court operational data including eCourt Tyler jury and internal sources; responses due May 13 2026 through Bonfire</x:v>
+        <x:v>Public Bonfire/GovTribe sources for SP-2026-0010 say Placer Court seeks Power BI development services to update rebuild and modernize about 20 existing dashboards across court operational data including eCourt Tyler jury and internal sources; Bonfire close is May 13 2026 at 5:00 PM Pacific</x:v>
       </x:c>
       <x:c r="J78" t="str">
         <x:v>Power BI dashboard modernization QA/UAT support</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>monitor_portal_qualified</x:v>
+        <x:v>prepared_portal_packet</x:v>
       </x:c>
       <x:c r="L78" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M78" t="str">
-        <x:v>Portal-only path; prepare only if Bonfire account/access is available or if a prime/subcontractor path appears; do not email unsolicited</x:v>
+        <x:v>Portal-only path; use prepared packet only through Bonfire or selected-vendor/subcontract path after reviewing required forms, insurance/vendor requirements, AI disclosure, and submission checklist; do not send casual email</x:v>
       </x:c>
       <x:c r="N78" t="str">
         <x:v>2026-05-12</x:v>
       </x:c>
       <x:c r="O78" t="str">
-        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/sp-2026-0010-power-bi-development-services-for-placer-court-sp20260010</x:v>
+        <x:v>placer-powerbi-qa-sidecar.html; outputs/codex10k/placer_powerbi_qa_uat_sidecar_proposal.pdf; docs/placer-bonfire-submission-notes.md; https://www.placer.courts.ca.gov/general-information/procurement; https://lacourt.bonfirehub.com/portal/?tab=openOpportunities; https://govtribe.com/opportunity/state-local-contract-opportunity/sp-2026-0010-power-bi-development-services-for-placer-court-sp20260010</x:v>
       </x:c>
       <x:c r="P78" t="str">
-        <x:v>Non-n8n analytics/data lane; likely requires formal portal response, insurance, business licensing, and procurement forms; best as portal-ready packet or subcontracted QA/UAT workstream</x:v>
+        <x:v>Non-n8n analytics/data lane; prepared USD 18500 Power BI QA/UAT/data-validation/handoff sidecar. Likely requires Bonfire account, formal portal response, business licensing, insurance, and procurement forms; best as portal-ready packet or selected-vendor/subcontract support</x:v>
       </x:c>
     </x:row>
     <x:row r="79">

</xml_diff>

<commit_message>
Prepare RRC Salesforce support packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rba9cd545e0ff48fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Ra10f7261f1704caf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R33cf8727c82042aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R0d1bbacf399e436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R77908f77fbc34995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rc5a0296a91ca408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R4fd80fd7684b4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R877f20326674415d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4275,28 +4275,28 @@
         <x:v>Salesforce implementation QA</x:v>
       </x:c>
       <x:c r="I79" t="str">
-        <x:v>Public sources for RFO 455-26-1018 say RRC seeks Salesforce and tools implementation services and support across Salesforce platform modernization and related tools; responses due May 19 2026 via Texas procurement channels</x:v>
+        <x:v>Public RFO materials for 455-26-1018 say RRC seeks Salesforce and tools implementation services and support across requirements, Salesforce configuration/development, data migration, integrations, testing, UAT, accessibility, training, documentation, and release support; responses due May 19 2026 at 2:00 PM Central</x:v>
       </x:c>
       <x:c r="J79" t="str">
-        <x:v>Salesforce implementation QA and requirements traceability sidecar</x:v>
+        <x:v>Salesforce QA/UAT migration-validation support slice</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>monitor_portal_qualified</x:v>
+        <x:v>prepared_subcontract_packet</x:v>
       </x:c>
       <x:c r="L79" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M79" t="str">
-        <x:v>Portal/procurement path; do not send as casual outreach; if pursuing, prepare subcontractor/QA packet around requirements traceability, migration QA, UAT scripts, dashboard acceptance, and defect triage</x:v>
+        <x:v>Do not send as casual outreach; use prepared USD 22500 support packet only through a qualified prime/subcontract path or formally approved response workflow after reviewing mandatory forms, Texas authorization, HSP/VetHUB, insurance, pricing worksheet, and AI disclosure requirements</x:v>
       </x:c>
       <x:c r="N79" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O79" t="str">
-        <x:v>https://www.rrc.texas.gov/about-us/contract-management/solicitations/; https://www.txsmartbuy.gov/esbd/455-26-1018</x:v>
+        <x:v>rrc-salesforce-qa-sidecar.html; outputs/codex10k/rrc_salesforce_qa_support_slice_proposal.pdf; docs/rrc-salesforce-subcontract-notes.md; https://www.txsmartbuy.gov/esbd/455-26-1018</x:v>
       </x:c>
       <x:c r="P79" t="str">
-        <x:v>Non-n8n Salesforce/data migration lane; likely requires Texas procurement compliance and prime/vendor credentials; better as named QA specialist or subcontract support</x:v>
+        <x:v>Non-n8n public-sector Salesforce/data migration lane; best angle is named specialist support for requirements traceability, migration QA, UAT scripts, regression/accessibility checks, Jira/Copado release evidence, documentation, and training handoff beside a compliant prime</x:v>
       </x:c>
     </x:row>
     <x:row r="80">

</xml_diff>

<commit_message>
Prepare MSPD migration QA portal packet
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R77908f77fbc34995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rc5a0296a91ca408f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R4fd80fd7684b4fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R877f20326674415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R26f8ad9fa0d44f2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rec049d4134e3456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rb302067f959745cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R37d07b38d69849da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4310,43 +4310,43 @@
         <x:v>Codex10k</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Missouri Office of State Public Defender</x:v>
+        <x:v>Missouri State Public Defender</x:v>
       </x:c>
       <x:c r="E80" t="str">
         <x:v>procurement@mspd.mo.gov</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>MissouriBUYS / public procurement mirror</x:v>
+        <x:v>MissouriBUYS / MOVERS / public procurement mirror</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>https://missouribuys.mo.gov</x:v>
+        <x:v>https://missouribuys.mo.gov/bid-board/movers</x:v>
       </x:c>
       <x:c r="H80" t="str">
         <x:v>Case-management migration QA</x:v>
       </x:c>
       <x:c r="I80" t="str">
-        <x:v>Public sources for MSPD 0000000003SL say Missouri State Public Defender seeks an integrated public defense management system covering case management, portals, court integrations, workflow automation, analytics, HCL Notes/Domino migration, and statewide rollout; proposals due June 30 2026 via MissouriBUYS</x:v>
+        <x:v>Public summaries for MSPD 0000000003SL describe an Integrated Public Defense Management System covering case management, portals, integrations, workflow automation, analytics, document intelligence, HCL Notes/Domino migration, UAT, training, and stabilization; responses due June 30 2026 at 5:00 PM Central through MissouriBUYS/MOVERS</x:v>
       </x:c>
       <x:c r="J80" t="str">
-        <x:v>Migration and implementation QA sidecar</x:v>
+        <x:v>Migration QA/UAT stabilization support slice</x:v>
       </x:c>
       <x:c r="K80" t="str">
-        <x:v>monitor_portal_qualified</x:v>
+        <x:v>prepared_portal_packet</x:v>
       </x:c>
       <x:c r="L80" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M80" t="str">
-        <x:v>Portal/procurement path with large prime scope; prepare only as subcontractor/QA sidecar unless full vendor team appears</x:v>
+        <x:v>Do not send as casual outreach; use prepared USD 28500 support packet only through MissouriBUYS/MOVERS, a qualified prime/subcontract path, or formally approved procurement workflow after reviewing supplier registration, required exhibits, insurance/security obligations, pricing schedules, and AI/disclosure requirements</x:v>
       </x:c>
       <x:c r="N80" t="str">
         <x:v>2026-05-20</x:v>
       </x:c>
       <x:c r="O80" t="str">
-        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/request-for-proposal-rfp-for-an-integrated-public-defense-management-system-300000235023766</x:v>
+        <x:v>mspd-case-migration-qa-sidecar.html; outputs/codex10k/mspd_case_migration_qa_support_slice_proposal.pdf; docs/mspd-case-management-subcontract-notes.md; https://govtribe.com/opportunity/state-local-contract-opportunity/request-for-proposal-rfp-for-an-integrated-public-defense-management-system-300000235023766; https://missouribuys.mo.gov/bid-board/movers</x:v>
       </x:c>
       <x:c r="P80" t="str">
-        <x:v>Non-n8n public-sector migration lane; strong fit for migration risk register, sample data validation, UAT/go-live templates, weekly status/reporting pack; too large for solo prime</x:v>
+        <x:v>Non-n8n public-sector migration lane; best angle is named specialist support for legacy migration QA, requirements traceability, UAT scripts, defect retest, reporting readiness, cutover evidence, and stabilization beside a compliant prime</x:v>
       </x:c>
     </x:row>
     <x:row r="81">

</xml_diff>

<commit_message>
Log Baxter outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R26f8ad9fa0d44f2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rec049d4134e3456f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rb302067f959745cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R37d07b38d69849da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R852bc827a75c4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Re6b1063511044286"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R776ca1d39e6646a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbf5ac05b57e044ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>76</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4399,6 +4399,56 @@
         <x:v>Sent USD 12000 limited multilingual/accessibility/content-migration QA sidecar with PDF attachment after cadence gate returned allowed and public page/PDF returned 200; not a full redesign-prime proposal, hosting proposal, CMS license, legal accessibility certification, or long-term maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>C10K-080</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>Baxter State Park Authority</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>nava.tabak@baxterstatepark.org</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Official RFP PDF / electronic proposal email</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>https://baxterstatepark.org/wp-content/uploads/2026/04/BSP-Request-for-Proposals-for-web-design-host-maintain-Apr-2026.docx.pdf</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>State park website launch QA</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>Official April 6 2026 RFP requests design of a new website plus hosting and technical maintenance with approximately 45 pages, ecommerce, search, semantic tags, ADA Title II web/mobile accessibility, responsive design, pre-production environment, CMS, transition support, performance testing, owner rights, and 365-day support models; electronic proposals due May 20 2026 to Nava Tabak</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>ADA/migration/performance/launch-readiness QA sidecar</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M82" t="str">
+        <x:v>Watch for RFP response/addenda registration; if positive, request procurement path, staging/vendor timeline, proposed structure, representative ecommerce/forms/search paths, preferred tracker format, and payment path</x:v>
+      </x:c>
+      <x:c r="N82" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O82" t="str">
+        <x:v>gmail:19e10a5e7c318c9b; baxter-website-launch-qa-sidecar.html; outputs/codex10k/baxter_website_launch_qa_sidecar_proposal.pdf; https://anonymusk7.github.io/codex10k-workflow-recovery/baxter-website-launch-qa-sidecar.html?v=baxter1</x:v>
+      </x:c>
+      <x:c r="P82" t="str">
+        <x:v>Sent USD 8500 limited ADA/migration/performance/launch-readiness QA sidecar with PDF attachment after cadence gate returned allowed and public page/PDF returned 200; not a full design-prime proposal, hosting proposal, CMS license, legal accessibility certification, or long-term maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Log Harford outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R852bc827a75c4526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Re6b1063511044286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R776ca1d39e6646a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbf5ac05b57e044ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a4fe699f1104cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R3f918011f84049d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R9e64c202e1af47be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R651d16ecf49b4f56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>77</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4449,6 +4449,56 @@
         <x:v>Sent USD 8500 limited ADA/migration/performance/launch-readiness QA sidecar with PDF attachment after cadence gate returned allowed and public page/PDF returned 200; not a full design-prime proposal, hosting proposal, CMS license, legal accessibility certification, or long-term maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>C10K-081</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>Harford County Public Schools</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>sara.rowe@hcps.org</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>Official procurement RFP / questions email</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>https://www.hcps.org/webfiles/WebFilesHandler.ashx?id=8727</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>K-12 transportation data readiness QA</x:v>
+      </x:c>
+      <x:c r="I83" t="str">
+        <x:v>Public RFP 26-SR-014 seeks Bus Routing, Fleet Management, GPS, and School Planning Solutions; subagent found procurement contact Sara Rowe and formal proposal path. Strong fit for limited routing data readiness, GPS validation samples, acceptance testing, issue register, and cutover evidence beside the primary solution vendor; questions due May 19 2026 and proposals due June 10 2026</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>Routing data readiness and acceptance QA support question</x:v>
+      </x:c>
+      <x:c r="K83" t="str">
+        <x:v>contacted_procurement_question</x:v>
+      </x:c>
+      <x:c r="L83" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M83" t="str">
+        <x:v>Watch for procurement response; if positive, follow the instructed formal path or selected-vendor route and request only sample/anonymized data, route-data field list, GPS validation expectations, acceptance-test format, and procurement/payment path</x:v>
+      </x:c>
+      <x:c r="N83" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O83" t="str">
+        <x:v>gmail:19e10c2baf1299e8; harford-routing-data-qa-sidecar.html; outputs/codex10k/harford_routing_data_qa_support_question.pdf; https://anonymusk7.github.io/codex10k-workflow-recovery/harford-routing-data-qa-sidecar.html?v=harford1</x:v>
+      </x:c>
+      <x:c r="P83" t="str">
+        <x:v>Sent USD 9500 limited routing data readiness and acceptance QA support question with PDF attachment after cadence gate returned allowed and manual 30-minute extra-send gap cleared; not a routing/fleet/GPS software bid, implementation-prime proposal, legal/privacy advice, or ongoing system maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Log Prince George parking outreach send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a4fe699f1104cca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R3f918011f84049d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R9e64c202e1af47be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R651d16ecf49b4f56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4250c5edebb3443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rda50023e806842af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R0cd3f782f3a6430a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R63505c4f74804de3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4499,6 +4499,56 @@
         <x:v>Sent USD 9500 limited routing data readiness and acceptance QA support question with PDF attachment after cadence gate returned allowed and manual 30-minute extra-send gap cleared; not a routing/fleet/GPS software bid, implementation-prime proposal, legal/privacy advice, or ongoing system maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>C10K-083</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Revenue Authority of Prince George's County</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>RVA-PMS.RFP@co.pg.md.us</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>Official solicitation page / electronic proposal email</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>https://www.princegeorgescountymd.gov/departments-offices/revenue-authority/solicitations</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>Parking management data migration QA</x:v>
+      </x:c>
+      <x:c r="I84" t="str">
+        <x:v>Official Revenue Authority solicitation for RVA-PMS-04-2026 Cloud-Based Parking Management System has electronic proposals due June 1 2026 at 2:00 PM EST. RFP scope includes cloud PMS, enforcement, citations, permits, payments, reporting, integrations, data migration, testing, training, BI dashboards, revenue analysis, forecasting, spatial mapping, and integrations such as LPR, PayLock, ERP/financial systems, Tyler/Court, Salesforce/311 CRM, collections, and DMV lookup</x:v>
+      </x:c>
+      <x:c r="J84" t="str">
+        <x:v>Parking data migration and integration acceptance QA support slice</x:v>
+      </x:c>
+      <x:c r="K84" t="str">
+        <x:v>contacted_fixed_scope</x:v>
+      </x:c>
+      <x:c r="L84" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M84" t="str">
+        <x:v>Watch for procurement response; if positive, request instructed formal path or selected-prime/subcontract path plus sample/anonymized records, integration list, reporting acceptance criteria, preferred UAT tracker format, and procurement/payment path</x:v>
+      </x:c>
+      <x:c r="N84" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O84" t="str">
+        <x:v>gmail:19e10e01ea3147ae; pgc-parking-data-qa-sidecar.html; outputs/codex10k/pgc_parking_data_qa_support_slice.pdf; https://anonymusk7.github.io/codex10k-workflow-recovery/pgc-parking-data-qa-sidecar.html?v=pgc1</x:v>
+      </x:c>
+      <x:c r="P84" t="str">
+        <x:v>Sent USD 14500 limited parking data migration and integration acceptance QA support slice with PDF attachment after cadence gate returned allowed and manual 30-minute extra-send gap cleared; not the full cloud PMS, hardware, LPR, enforcement platform, legal compliance, cyber insurance package, or ongoing maintenance contract</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Prepare Codex10k draft email batch
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4250c5edebb3443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rda50023e806842af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R0cd3f782f3a6430a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R63505c4f74804de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf5e0f2dfc0174218"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rbefafac512d543e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R964aa28fbe2b448d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Red927650109e40f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>79</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4549,6 +4549,1006 @@
         <x:v>Sent USD 14500 limited parking data migration and integration acceptance QA support slice with PDF attachment after cadence gate returned allowed and manual 30-minute extra-send gap cleared; not the full cloud PMS, hardware, LPR, enforcement platform, legal compliance, cyber insurance package, or ongoing maintenance contract</x:v>
       </x:c>
     </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>C10K-084</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>BakerRipley</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>abrown@bakerripley.org</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>https://bakerripley.org/get-involved/become-a-vendor/</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>Salesforce services support</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>The main RFP is for Salesforce professional services; the useful lane here is implementation QA, migration sampling, and UAT evidence beside a qualified Salesforce team.</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>Salesforce implementation QA and UAT support sidecar</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L85" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M85" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N85" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O85" t="str">
+        <x:v>c10k-084-bakerripley.html; outputs/codex10k/draft-batch/c10k-084-bakerripley.pdf; outputs/codex10k/draft-batch/c10k-084-bakerripley.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-084-bakerripley.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P85" t="str">
+        <x:v>Mandatory vendor conference risk. This draft asks eligibility before proposing work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>C10K-085</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Connecticut Auditors of Public Accounts</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Sandra.DeLaCruz@cga.ct.gov; vincent.filippa@ctauditors.gov</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/2026-01-apa-microsoft-sharepoint-maintenance-rfp-202601apa</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>SharePoint maintenance support</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>The RFP maps well to SharePoint workflow maintenance, permission review, template QA, and repeatable support evidence.</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>SharePoint workflow QA and maintenance support slice</x:v>
+      </x:c>
+      <x:c r="K86" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L86" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N86" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O86" t="str">
+        <x:v>c10k-085-connecticut-auditors-of-public-accounts.html; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.pdf; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-085-connecticut-auditors-of-public-accounts.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P86" t="str">
+        <x:v>Email is appropriate, but Sandra is the inquiry contact; proposal/submission goes to Vincent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>C10K-086</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Maine Community College System</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>sfortin@mainecc.edu</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>https://www.mccs.me.edu/request-for-proposals/</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>IAM rollout support</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>IAM rollout risk often concentrates around role mapping, provisioning/deprovisioning tests, exception handling, and staff handoff.</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>IAM role validation and rollout QA support</x:v>
+      </x:c>
+      <x:c r="K87" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L87" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M87" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N87" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O87" t="str">
+        <x:v>c10k-086-maine-community-college-system.html; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.pdf; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-086-maine-community-college-system.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P87" t="str">
+        <x:v>Email submission is allowed, but questions deadline passed; keep this as a support component, not a substantive RFP question.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>C10K-087</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>American Battle Monuments Commission</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>nerenga@abmc.gov</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>https://www.abmc.gov/rfp/74330226r0044-human-resources-information-system/</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>HRIS implementation support</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>The full HRIS response is formal, but a compact migration/UAT support slice can strengthen the implementation evidence if ABMC or a prime uses specialist support.</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>HRIS migration and acceptance QA support</x:v>
+      </x:c>
+      <x:c r="K88" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N88" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O88" t="str">
+        <x:v>c10k-087-american-battle-monuments-commission.html; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.pdf; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-087-american-battle-monuments-commission.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P88" t="str">
+        <x:v>Federal HRIS. Avoid PII and avoid implying this is the full HRIS proposal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>C10K-088</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Friends of Springfield Art Museum</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>kate.francis@springfieldmo.gov</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>https://sgfmuseum.org/m/newsflash/Home/Detail/228</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>Museum CRM support</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>The RFQ needs CRM judgment; data mapping, dedupe, import sampling, UAT scripts, and launch evidence are a practical fixed support lane.</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>Museum CRM data migration and acceptance QA support</x:v>
+      </x:c>
+      <x:c r="K89" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L89" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M89" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N89" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O89" t="str">
+        <x:v>c10k-088-friends-of-springfield-art-museum.html; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.pdf; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-088-friends-of-springfield-art-museum.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P89" t="str">
+        <x:v>Email is allowed. Keep formal, RFQ-specific, and do not claim platform-prime qualifications.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>C10K-089</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Town of Hillsborough</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>dbelcik@hillsborough.net</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>https://www.hillsborough.net/207/Request-for-Proposals</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>Municipal data support</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>The support lane is data, GIS, issue tracking, public-facing deliverable QA, and handoff evidence beside licensed professionals.</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>GIS/data workflow QA and deliverable support slice</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N90" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O90" t="str">
+        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P90" t="str">
+        <x:v>Do not imply engineering credentials. Email is appropriate only as a support/teaming question.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>C10K-090</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Society of St. Vincent de Paul Cincinnati</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>ajones@svdpcincinnati.org; andy.ey@svdpcincinnati.org</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>https://www.svdpcincinnati.org/wp-content/uploads/2026/04/RFP-for-St.-Vincent-de-Paul-Website.pdf</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>Nonprofit website support</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>The RFP is mission-critical: donor trust, volunteer conversion, service navigation, and accessible content all need structured QA before launch.</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>Website launch QA, accessibility, and donor-path support</x:v>
+      </x:c>
+      <x:c r="K91" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N91" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O91" t="str">
+        <x:v>c10k-090-society-of-st-vincent-de-paul-cincinnati.html; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.pdf; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-090-society-of-st-vincent-de-paul-cincinnati.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P91" t="str">
+        <x:v>Direct email is available. Local-firm preference exists, so keep this as support-sidecar unless bidding as prime.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>C10K-091</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Northumberland Humane Society</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>campaigndirector@northumberlandhs.com</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>https://www.northumberlandhs.com/s/Website-Development_RFP_V1-1.pdf</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>Animal welfare website support</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>The website needs to support adoption interest, campaign storytelling, CanadaHelps, DonorPerfect, Mailchimp, mobile access, and accessible public content.</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>Donation, adoption, and campaign website QA support</x:v>
+      </x:c>
+      <x:c r="K92" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N92" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O92" t="str">
+        <x:v>c10k-091-northumberland-humane-society.html; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.pdf; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-091-northumberland-humane-society.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P92" t="str">
+        <x:v>Ontario/local vendor preference. Keep as support-sidecar and do not imply local status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>C10K-092</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Institute of International Education</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Arowland@iie.org</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>https://www.iie.org/get-involved/procurement-subaward-and-consultant-opportunities/solicitations-for-goods-and-services/</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>Education website maintenance support</x:v>
+      </x:c>
+      <x:c r="I93" t="str">
+        <x:v>The RFP calls for website maintenance, enhancement, quarterly checks, broken-link/form testing, analytics reporting, access-controlled content, and responsiveness standards.</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>Fulbright Scholar website maintenance QA and accessibility support</x:v>
+      </x:c>
+      <x:c r="K93" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L93" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M93" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N93" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O93" t="str">
+        <x:v>c10k-092-institute-of-international-education.html; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.pdf; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-092-institute-of-international-education.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P93" t="str">
+        <x:v>Full-service RFP. Keep as support slice unless user can submit full qualified proposal.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>C10K-093</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>THRIVE Victoria</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>development@thrivevictoria.org</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>https://thrivevictoria.org/jobs/website-designer/</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>Nonprofit campaign website support</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>The RFP has clear dual-user journeys: donors/funders and clients/youth/families. That makes structured path testing, accessibility, privacy-safe forms, and CMS handoff especially important.</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>Youth-services website QA and campaign-readiness support</x:v>
+      </x:c>
+      <x:c r="K94" t="str">
+        <x:v>gmail_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L94" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M94" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N94" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O94" t="str">
+        <x:v>c10k-093-thrive-victoria.html; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.pdf; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-093-thrive-victoria.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P94" t="str">
+        <x:v>Direct email proposal path. Canadian nonprofit; quote in USD for Codex10k tracking but buyer budget is CAD.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>C10K-094</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Baxter State Park Authority</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>nava.tabak@baxterstatepark.org</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/baxter-website-launch-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>State park website support</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>Baxter ADA/migration launch QA follow-up</x:v>
+      </x:c>
+      <x:c r="K95" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L95" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N95" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O95" t="str">
+        <x:v>c10k-094-baxter-state-park-authority.html; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.pdf; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-094-baxter-state-park-authority.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P95" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>C10K-095</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>Harford County Public Schools</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>sara.rowe@hcps.org</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/harford-routing-data-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>K-12 routing data support</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>Harford routing data QA follow-up</x:v>
+      </x:c>
+      <x:c r="K96" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L96" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M96" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N96" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O96" t="str">
+        <x:v>c10k-095-harford-county-public-schools.html; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.pdf; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-095-harford-county-public-schools.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P96" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>C10K-096</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Revenue Authority of Prince George's County</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>RVA-PMS.RFP@co.pg.md.us</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/pgc-parking-data-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Parking data support</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Parking PMS migration QA follow-up</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M97" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N97" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O97" t="str">
+        <x:v>c10k-096-revenue-authority-of-prince-george-s-county.html; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.pdf; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-096-revenue-authority-of-prince-george-s-county.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P97" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>C10K-097</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Napa Valley Transportation Authority</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>procurements@nvta.ca.gov; rcoombs@nvta.ca.gov</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/nvta-ada-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>ADA website QA support</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>NVTA ADA website QA follow-up</x:v>
+      </x:c>
+      <x:c r="K98" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L98" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M98" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N98" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O98" t="str">
+        <x:v>c10k-097-napa-valley-transportation-authority.html; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.pdf; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-097-napa-valley-transportation-authority.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P98" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>C10K-098</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Town of Duck</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>knickens@ducknc.gov</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/duck-ada-launch-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>Municipal website launch support</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>Town of Duck launch QA follow-up</x:v>
+      </x:c>
+      <x:c r="K99" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L99" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M99" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N99" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O99" t="str">
+        <x:v>c10k-098-town-of-duck.html; outputs/codex10k/draft-batch/c10k-098-town-of-duck.pdf; outputs/codex10k/draft-batch/c10k-098-town-of-duck.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-098-town-of-duck.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P99" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>C10K-099</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Ely Area Tourism Bureau</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>jess@rootbeerlady.com</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/ely-migration-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Tourism website migration support</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>Ely tourism migration QA follow-up</x:v>
+      </x:c>
+      <x:c r="K100" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N100" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O100" t="str">
+        <x:v>c10k-099-ely-area-tourism-bureau.html; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.pdf; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-099-ely-area-tourism-bureau.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P100" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>C10K-100</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Hiawatha Academies</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>kgroves@hiawathaacademies.org</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/hiawatha-school-website-qa-sidecar.html</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>School website QA support</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>Hiawatha multilingual website QA follow-up</x:v>
+      </x:c>
+      <x:c r="K101" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L101" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M101" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N101" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O101" t="str">
+        <x:v>c10k-100-hiawatha-academies.html; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.pdf; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-100-hiawatha-academies.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P101" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>C10K-101</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>3D Walkabout</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>tim@3dwalkabout.com.au</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/3dwalkabout-hubspot-clickup.html</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>CRM automation support</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>3D Walkabout HubSpot-ClickUp sprint follow-up</x:v>
+      </x:c>
+      <x:c r="K102" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L102" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M102" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N102" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O102" t="str">
+        <x:v>c10k-101-3d-walkabout.html; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.pdf; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-101-3d-walkabout.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P102" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>C10K-102</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>SnipeAgent</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>contact@snipeagent.ai</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/snipeagent-sms-automation.html</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>SMS automation architecture support</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>SnipeAgent architecture pass follow-up</x:v>
+      </x:c>
+      <x:c r="K103" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L103" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M103" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N103" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O103" t="str">
+        <x:v>c10k-102-snipeagent.html; outputs/codex10k/draft-batch/c10k-102-snipeagent.pdf; outputs/codex10k/draft-batch/c10k-102-snipeagent.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-102-snipeagent.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P103" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>C10K-103</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Chek Creative</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>hello@chekcreative.com</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>Gmail draft packet / public source</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>https://anonymusk7.github.io/codex10k-workflow-recovery/chek-automation-partner-pilot.html</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>Automation agency support</x:v>
+      </x:c>
+      <x:c r="I104" t="str">
+        <x:v>This is already scoped around the buyer's public RFP, public support request, or previously sent packet.</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>Chek Creative automation pilot follow-up</x:v>
+      </x:c>
+      <x:c r="K104" t="str">
+        <x:v>followup_draft_packet_prepared</x:v>
+      </x:c>
+      <x:c r="L104" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M104" t="str">
+        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+      </x:c>
+      <x:c r="N104" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O104" t="str">
+        <x:v>c10k-103-chek-creative.html; outputs/codex10k/draft-batch/c10k-103-chek-creative.pdf; outputs/codex10k/draft-batch/c10k-103-chek-creative.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-103-chek-creative.html?v=draft1</x:v>
+      </x:c>
+      <x:c r="P104" t="str">
+        <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Log Gmail draft batch
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rf5e0f2dfc0174218"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rbefafac512d543e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R964aa28fbe2b448d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Red927650109e40f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R23f8d61136d749cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R75aa6fee9a114a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R3c583e49f94c4016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rc91bc0005c4b4588"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4581,19 +4581,19 @@
         <x:v>Salesforce implementation QA and UAT support sidecar</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L85" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M85" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N85" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O85" t="str">
-        <x:v>c10k-084-bakerripley.html; outputs/codex10k/draft-batch/c10k-084-bakerripley.pdf; outputs/codex10k/draft-batch/c10k-084-bakerripley.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-084-bakerripley.html?v=draft1</x:v>
+        <x:v>c10k-084-bakerripley.html; outputs/codex10k/draft-batch/c10k-084-bakerripley.pdf; outputs/codex10k/draft-batch/c10k-084-bakerripley.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-084-bakerripley.html?v=draft1; gmail_draft:r7718642615731016285; gmail_msg:19e1131cdbe3bdaf</x:v>
       </x:c>
       <x:c r="P85" t="str">
         <x:v>Mandatory vendor conference risk. This draft asks eligibility before proposing work.</x:v>
@@ -4631,19 +4631,19 @@
         <x:v>SharePoint workflow QA and maintenance support slice</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L86" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M86" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N86" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O86" t="str">
-        <x:v>c10k-085-connecticut-auditors-of-public-accounts.html; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.pdf; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-085-connecticut-auditors-of-public-accounts.html?v=draft1</x:v>
+        <x:v>c10k-085-connecticut-auditors-of-public-accounts.html; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.pdf; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-085-connecticut-auditors-of-public-accounts.html?v=draft1; gmail_draft:r-5424769604189818739; gmail_msg:19e11323eb29966e</x:v>
       </x:c>
       <x:c r="P86" t="str">
         <x:v>Email is appropriate, but Sandra is the inquiry contact; proposal/submission goes to Vincent.</x:v>
@@ -4681,19 +4681,19 @@
         <x:v>IAM role validation and rollout QA support</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L87" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N87" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O87" t="str">
-        <x:v>c10k-086-maine-community-college-system.html; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.pdf; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-086-maine-community-college-system.html?v=draft1</x:v>
+        <x:v>c10k-086-maine-community-college-system.html; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.pdf; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-086-maine-community-college-system.html?v=draft1; gmail_draft:r7792718751307555089; gmail_msg:19e113286e3d869b</x:v>
       </x:c>
       <x:c r="P87" t="str">
         <x:v>Email submission is allowed, but questions deadline passed; keep this as a support component, not a substantive RFP question.</x:v>
@@ -4731,19 +4731,19 @@
         <x:v>HRIS migration and acceptance QA support</x:v>
       </x:c>
       <x:c r="K88" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L88" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M88" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N88" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O88" t="str">
-        <x:v>c10k-087-american-battle-monuments-commission.html; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.pdf; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-087-american-battle-monuments-commission.html?v=draft1</x:v>
+        <x:v>c10k-087-american-battle-monuments-commission.html; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.pdf; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-087-american-battle-monuments-commission.html?v=draft1; gmail_draft:r8757273967754748544; gmail_msg:19e1132cd3f3895f</x:v>
       </x:c>
       <x:c r="P88" t="str">
         <x:v>Federal HRIS. Avoid PII and avoid implying this is the full HRIS proposal.</x:v>
@@ -4781,19 +4781,19 @@
         <x:v>Museum CRM data migration and acceptance QA support</x:v>
       </x:c>
       <x:c r="K89" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L89" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M89" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N89" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O89" t="str">
-        <x:v>c10k-088-friends-of-springfield-art-museum.html; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.pdf; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-088-friends-of-springfield-art-museum.html?v=draft1</x:v>
+        <x:v>c10k-088-friends-of-springfield-art-museum.html; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.pdf; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-088-friends-of-springfield-art-museum.html?v=draft1; gmail_draft:r-516733945645526600; gmail_msg:19e113327b7d8fb3</x:v>
       </x:c>
       <x:c r="P89" t="str">
         <x:v>Email is allowed. Keep formal, RFQ-specific, and do not claim platform-prime qualifications.</x:v>
@@ -4831,19 +4831,19 @@
         <x:v>GIS/data workflow QA and deliverable support slice</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L90" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M90" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N90" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O90" t="str">
-        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1</x:v>
+        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1; gmail_draft:r-3371871953269203560; gmail_msg:19e11337718ef02e</x:v>
       </x:c>
       <x:c r="P90" t="str">
         <x:v>Do not imply engineering credentials. Email is appropriate only as a support/teaming question.</x:v>
@@ -4881,19 +4881,19 @@
         <x:v>Website launch QA, accessibility, and donor-path support</x:v>
       </x:c>
       <x:c r="K91" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L91" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M91" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N91" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O91" t="str">
-        <x:v>c10k-090-society-of-st-vincent-de-paul-cincinnati.html; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.pdf; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-090-society-of-st-vincent-de-paul-cincinnati.html?v=draft1</x:v>
+        <x:v>c10k-090-society-of-st-vincent-de-paul-cincinnati.html; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.pdf; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-090-society-of-st-vincent-de-paul-cincinnati.html?v=draft1; gmail_draft:r1477712879751866611; gmail_msg:19e1133bd871a403</x:v>
       </x:c>
       <x:c r="P91" t="str">
         <x:v>Direct email is available. Local-firm preference exists, so keep this as support-sidecar unless bidding as prime.</x:v>
@@ -4931,19 +4931,19 @@
         <x:v>Donation, adoption, and campaign website QA support</x:v>
       </x:c>
       <x:c r="K92" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L92" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M92" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N92" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O92" t="str">
-        <x:v>c10k-091-northumberland-humane-society.html; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.pdf; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-091-northumberland-humane-society.html?v=draft1</x:v>
+        <x:v>c10k-091-northumberland-humane-society.html; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.pdf; outputs/codex10k/draft-batch/c10k-091-northumberland-humane-society.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-091-northumberland-humane-society.html?v=draft1; gmail_draft:r9137065922616610769; gmail_msg:19e11340feabaf61</x:v>
       </x:c>
       <x:c r="P92" t="str">
         <x:v>Ontario/local vendor preference. Keep as support-sidecar and do not imply local status.</x:v>
@@ -4981,19 +4981,19 @@
         <x:v>Fulbright Scholar website maintenance QA and accessibility support</x:v>
       </x:c>
       <x:c r="K93" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L93" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M93" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N93" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O93" t="str">
-        <x:v>c10k-092-institute-of-international-education.html; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.pdf; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-092-institute-of-international-education.html?v=draft1</x:v>
+        <x:v>c10k-092-institute-of-international-education.html; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.pdf; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-092-institute-of-international-education.html?v=draft1; gmail_draft:r-4264919839455923807; gmail_msg:19e11345f9759c29</x:v>
       </x:c>
       <x:c r="P93" t="str">
         <x:v>Full-service RFP. Keep as support slice unless user can submit full qualified proposal.</x:v>
@@ -5031,19 +5031,19 @@
         <x:v>Youth-services website QA and campaign-readiness support</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>gmail_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L94" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M94" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N94" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O94" t="str">
-        <x:v>c10k-093-thrive-victoria.html; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.pdf; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-093-thrive-victoria.html?v=draft1</x:v>
+        <x:v>c10k-093-thrive-victoria.html; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.pdf; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-093-thrive-victoria.html?v=draft1; gmail_draft:r341758721023828887; gmail_msg:19e1134e72b60be7</x:v>
       </x:c>
       <x:c r="P94" t="str">
         <x:v>Direct email proposal path. Canadian nonprofit; quote in USD for Codex10k tracking but buyer budget is CAD.</x:v>
@@ -5081,19 +5081,19 @@
         <x:v>Baxter ADA/migration launch QA follow-up</x:v>
       </x:c>
       <x:c r="K95" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L95" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M95" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N95" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O95" t="str">
-        <x:v>c10k-094-baxter-state-park-authority.html; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.pdf; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-094-baxter-state-park-authority.html?v=draft1</x:v>
+        <x:v>c10k-094-baxter-state-park-authority.html; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.pdf; outputs/codex10k/draft-batch/c10k-094-baxter-state-park-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-094-baxter-state-park-authority.html?v=draft1; gmail_draft:r5353432031169205359; gmail_msg:19e113580f66531a</x:v>
       </x:c>
       <x:c r="P95" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5131,19 +5131,19 @@
         <x:v>Harford routing data QA follow-up</x:v>
       </x:c>
       <x:c r="K96" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L96" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M96" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N96" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O96" t="str">
-        <x:v>c10k-095-harford-county-public-schools.html; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.pdf; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-095-harford-county-public-schools.html?v=draft1</x:v>
+        <x:v>c10k-095-harford-county-public-schools.html; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.pdf; outputs/codex10k/draft-batch/c10k-095-harford-county-public-schools.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-095-harford-county-public-schools.html?v=draft1; gmail_draft:r3100201977837495910; gmail_msg:19e1135ccf33002a</x:v>
       </x:c>
       <x:c r="P96" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5181,19 +5181,19 @@
         <x:v>Parking PMS migration QA follow-up</x:v>
       </x:c>
       <x:c r="K97" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L97" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M97" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N97" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O97" t="str">
-        <x:v>c10k-096-revenue-authority-of-prince-george-s-county.html; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.pdf; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-096-revenue-authority-of-prince-george-s-county.html?v=draft1</x:v>
+        <x:v>c10k-096-revenue-authority-of-prince-george-s-county.html; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.pdf; outputs/codex10k/draft-batch/c10k-096-revenue-authority-of-prince-george-s-county.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-096-revenue-authority-of-prince-george-s-county.html?v=draft1; gmail_draft:r5521619101680114811; gmail_msg:19e113610ef1cc11</x:v>
       </x:c>
       <x:c r="P97" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5231,19 +5231,19 @@
         <x:v>NVTA ADA website QA follow-up</x:v>
       </x:c>
       <x:c r="K98" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L98" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M98" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N98" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O98" t="str">
-        <x:v>c10k-097-napa-valley-transportation-authority.html; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.pdf; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-097-napa-valley-transportation-authority.html?v=draft1</x:v>
+        <x:v>c10k-097-napa-valley-transportation-authority.html; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.pdf; outputs/codex10k/draft-batch/c10k-097-napa-valley-transportation-authority.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-097-napa-valley-transportation-authority.html?v=draft1; gmail_draft:r907155150484054466; gmail_msg:19e11364fd65bdc7</x:v>
       </x:c>
       <x:c r="P98" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5281,19 +5281,19 @@
         <x:v>Town of Duck launch QA follow-up</x:v>
       </x:c>
       <x:c r="K99" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L99" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M99" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N99" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O99" t="str">
-        <x:v>c10k-098-town-of-duck.html; outputs/codex10k/draft-batch/c10k-098-town-of-duck.pdf; outputs/codex10k/draft-batch/c10k-098-town-of-duck.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-098-town-of-duck.html?v=draft1</x:v>
+        <x:v>c10k-098-town-of-duck.html; outputs/codex10k/draft-batch/c10k-098-town-of-duck.pdf; outputs/codex10k/draft-batch/c10k-098-town-of-duck.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-098-town-of-duck.html?v=draft1; gmail_draft:r3606409848104572723; gmail_msg:19e1136991db974d</x:v>
       </x:c>
       <x:c r="P99" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5331,19 +5331,19 @@
         <x:v>Ely tourism migration QA follow-up</x:v>
       </x:c>
       <x:c r="K100" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L100" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M100" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N100" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O100" t="str">
-        <x:v>c10k-099-ely-area-tourism-bureau.html; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.pdf; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-099-ely-area-tourism-bureau.html?v=draft1</x:v>
+        <x:v>c10k-099-ely-area-tourism-bureau.html; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.pdf; outputs/codex10k/draft-batch/c10k-099-ely-area-tourism-bureau.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-099-ely-area-tourism-bureau.html?v=draft1; gmail_draft:r-4234669480558694433; gmail_msg:19e1136df9736d9e</x:v>
       </x:c>
       <x:c r="P100" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5381,19 +5381,19 @@
         <x:v>Hiawatha multilingual website QA follow-up</x:v>
       </x:c>
       <x:c r="K101" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L101" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M101" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N101" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O101" t="str">
-        <x:v>c10k-100-hiawatha-academies.html; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.pdf; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-100-hiawatha-academies.html?v=draft1</x:v>
+        <x:v>c10k-100-hiawatha-academies.html; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.pdf; outputs/codex10k/draft-batch/c10k-100-hiawatha-academies.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-100-hiawatha-academies.html?v=draft1; gmail_draft:r3962797927973152463; gmail_msg:19e11372d0f5c8db</x:v>
       </x:c>
       <x:c r="P101" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5431,19 +5431,19 @@
         <x:v>3D Walkabout HubSpot-ClickUp sprint follow-up</x:v>
       </x:c>
       <x:c r="K102" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L102" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M102" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N102" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O102" t="str">
-        <x:v>c10k-101-3d-walkabout.html; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.pdf; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-101-3d-walkabout.html?v=draft1</x:v>
+        <x:v>c10k-101-3d-walkabout.html; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.pdf; outputs/codex10k/draft-batch/c10k-101-3d-walkabout.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-101-3d-walkabout.html?v=draft1; gmail_draft:r8198823679674218259; gmail_msg:19e113780da4b0c6</x:v>
       </x:c>
       <x:c r="P102" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5481,19 +5481,19 @@
         <x:v>SnipeAgent architecture pass follow-up</x:v>
       </x:c>
       <x:c r="K103" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L103" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M103" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N103" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O103" t="str">
-        <x:v>c10k-102-snipeagent.html; outputs/codex10k/draft-batch/c10k-102-snipeagent.pdf; outputs/codex10k/draft-batch/c10k-102-snipeagent.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-102-snipeagent.html?v=draft1</x:v>
+        <x:v>c10k-102-snipeagent.html; outputs/codex10k/draft-batch/c10k-102-snipeagent.pdf; outputs/codex10k/draft-batch/c10k-102-snipeagent.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-102-snipeagent.html?v=draft1; gmail_draft:r332576918970528924; gmail_msg:19e1137c0bd591c1</x:v>
       </x:c>
       <x:c r="P103" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
@@ -5531,19 +5531,19 @@
         <x:v>Chek Creative automation pilot follow-up</x:v>
       </x:c>
       <x:c r="K104" t="str">
-        <x:v>followup_draft_packet_prepared</x:v>
+        <x:v>gmail_draft_created_no_send</x:v>
       </x:c>
       <x:c r="L104" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M104" t="str">
-        <x:v>Review Gmail draft and send manually only if desired; do not use automated send cadence for this draft batch.</x:v>
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
       </x:c>
       <x:c r="N104" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O104" t="str">
-        <x:v>c10k-103-chek-creative.html; outputs/codex10k/draft-batch/c10k-103-chek-creative.pdf; outputs/codex10k/draft-batch/c10k-103-chek-creative.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-103-chek-creative.html?v=draft1</x:v>
+        <x:v>c10k-103-chek-creative.html; outputs/codex10k/draft-batch/c10k-103-chek-creative.pdf; outputs/codex10k/draft-batch/c10k-103-chek-creative.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-103-chek-creative.html?v=draft1; gmail_draft:r-3557540405541149303; gmail_msg:19e11382b690d1e5</x:v>
       </x:c>
       <x:c r="P104" t="str">
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>

</xml_diff>

<commit_message>
Log C10K-090 draft send
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R23f8d61136d749cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R75aa6fee9a114a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R3c583e49f94c4016"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rc91bc0005c4b4588"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9aae24fb60c44ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rb75bf004f5df4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R82f7abdb27374d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R7555dd0698704f20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4881,22 +4881,22 @@
         <x:v>Website launch QA, accessibility, and donor-path support</x:v>
       </x:c>
       <x:c r="K91" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L91" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M91" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and request billing/procurement path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N91" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O91" t="str">
-        <x:v>c10k-090-society-of-st-vincent-de-paul-cincinnati.html; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.pdf; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-090-society-of-st-vincent-de-paul-cincinnati.html?v=draft1; gmail_draft:r1477712879751866611; gmail_msg:19e1133bd871a403</x:v>
+        <x:v>c10k-090-society-of-st-vincent-de-paul-cincinnati.html; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.pdf; outputs/codex10k/draft-batch/c10k-090-society-of-st-vincent-de-paul-cincinnati.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-090-society-of-st-vincent-de-paul-cincinnati.html?v=draft1; gmail_draft:r1477712879751866611; gmail_msg:19e1133bd871a403; gmail_sent:19e1156ecebc569a</x:v>
       </x:c>
       <x:c r="P91" t="str">
-        <x:v>Direct email is available. Local-firm preference exists, so keep this as support-sidecar unless bidding as prime.</x:v>
+        <x:v>Sent from Gmail draft after user approved 7 highest-confidence drafts and raised May 10 cap to 20. Local-firm preference exists, so keep this as support-sidecar unless bidding as prime.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">

</xml_diff>

<commit_message>
Send seven Codex10k draft proposals
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9aae24fb60c44ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rb75bf004f5df4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R82f7abdb27374d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R7555dd0698704f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8d64cef1e09a4cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R1ee43fbe66274aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R6200f806ceec486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rb3404269fa9f42a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4631,22 +4631,22 @@
         <x:v>SharePoint workflow QA and maintenance support slice</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L86" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M86" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and follow the confirmed procurement recipient/path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N86" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O86" t="str">
-        <x:v>c10k-085-connecticut-auditors-of-public-accounts.html; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.pdf; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-085-connecticut-auditors-of-public-accounts.html?v=draft1; gmail_draft:r-5424769604189818739; gmail_msg:19e11323eb29966e</x:v>
+        <x:v>c10k-085-connecticut-auditors-of-public-accounts.html; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.pdf; outputs/codex10k/draft-batch/c10k-085-connecticut-auditors-of-public-accounts.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-085-connecticut-auditors-of-public-accounts.html?v=draft1; gmail_draft:r-5424769604189818739; gmail_msg:19e11323eb29966e; gmail_sent:19e1164ed277bac1</x:v>
       </x:c>
       <x:c r="P86" t="str">
-        <x:v>Email is appropriate, but Sandra is the inquiry contact; proposal/submission goes to Vincent.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Email is appropriate, but Sandra is the inquiry contact; proposal/submission goes to Vincent.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4681,22 +4681,22 @@
         <x:v>IAM role validation and rollout QA support</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L87" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm support-component eligibility before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N87" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O87" t="str">
-        <x:v>c10k-086-maine-community-college-system.html; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.pdf; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-086-maine-community-college-system.html?v=draft1; gmail_draft:r7792718751307555089; gmail_msg:19e113286e3d869b</x:v>
+        <x:v>c10k-086-maine-community-college-system.html; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.pdf; outputs/codex10k/draft-batch/c10k-086-maine-community-college-system.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-086-maine-community-college-system.html?v=draft1; gmail_draft:r7792718751307555089; gmail_msg:19e113286e3d869b; gmail_sent:19e1168efc6a0bf2</x:v>
       </x:c>
       <x:c r="P87" t="str">
-        <x:v>Email submission is allowed, but questions deadline passed; keep this as a support component, not a substantive RFP question.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Email submission is allowed, but questions deadline passed; keep this as a support component, not a substantive RFP question.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4781,22 +4781,22 @@
         <x:v>Museum CRM data migration and acceptance QA support</x:v>
       </x:c>
       <x:c r="K89" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L89" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M89" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm CRM QA support path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N89" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O89" t="str">
-        <x:v>c10k-088-friends-of-springfield-art-museum.html; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.pdf; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-088-friends-of-springfield-art-museum.html?v=draft1; gmail_draft:r-516733945645526600; gmail_msg:19e113327b7d8fb3</x:v>
+        <x:v>c10k-088-friends-of-springfield-art-museum.html; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.pdf; outputs/codex10k/draft-batch/c10k-088-friends-of-springfield-art-museum.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-088-friends-of-springfield-art-museum.html?v=draft1; gmail_draft:r-516733945645526600; gmail_msg:19e113327b7d8fb3; gmail_sent:19e1160e7651b392</x:v>
       </x:c>
       <x:c r="P89" t="str">
-        <x:v>Email is allowed. Keep formal, RFQ-specific, and do not claim platform-prime qualifications.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Keep formal, RFQ-specific, and do not claim platform-prime qualifications.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4831,22 +4831,22 @@
         <x:v>GIS/data workflow QA and deliverable support slice</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L90" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M90" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm support/teaming path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N90" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O90" t="str">
-        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1; gmail_draft:r-3371871953269203560; gmail_msg:19e11337718ef02e</x:v>
+        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1; gmail_draft:r-3371871953269203560; gmail_msg:19e11337718ef02e; gmail_sent:19e116d0b7e2a01a</x:v>
       </x:c>
       <x:c r="P90" t="str">
-        <x:v>Do not imply engineering credentials. Email is appropriate only as a support/teaming question.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Do not imply engineering credentials; support/teaming path only.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4981,22 +4981,22 @@
         <x:v>Fulbright Scholar website maintenance QA and accessibility support</x:v>
       </x:c>
       <x:c r="K93" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L93" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M93" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm formal support-slice path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N93" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O93" t="str">
-        <x:v>c10k-092-institute-of-international-education.html; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.pdf; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-092-institute-of-international-education.html?v=draft1; gmail_draft:r-4264919839455923807; gmail_msg:19e11345f9759c29</x:v>
+        <x:v>c10k-092-institute-of-international-education.html; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.pdf; outputs/codex10k/draft-batch/c10k-092-institute-of-international-education.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-092-institute-of-international-education.html?v=draft1; gmail_draft:r-4264919839455923807; gmail_msg:19e11345f9759c29; gmail_sent:19e115cdb8d63f15</x:v>
       </x:c>
       <x:c r="P93" t="str">
-        <x:v>Full-service RFP. Keep as support slice unless user can submit full qualified proposal.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Full-service RFP; keep as support slice unless user can submit full qualified proposal.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -5031,22 +5031,22 @@
         <x:v>Youth-services website QA and campaign-readiness support</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L94" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M94" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm USD/CAD billing path before any payment link/invoice</x:v>
       </x:c>
       <x:c r="N94" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O94" t="str">
-        <x:v>c10k-093-thrive-victoria.html; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.pdf; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-093-thrive-victoria.html?v=draft1; gmail_draft:r341758721023828887; gmail_msg:19e1134e72b60be7</x:v>
+        <x:v>c10k-093-thrive-victoria.html; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.pdf; outputs/codex10k/draft-batch/c10k-093-thrive-victoria.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-093-thrive-victoria.html?v=draft1; gmail_draft:r341758721023828887; gmail_msg:19e1134e72b60be7; gmail_sent:19e115910fe3140c</x:v>
       </x:c>
       <x:c r="P94" t="str">
-        <x:v>Direct email proposal path. Canadian nonprofit; quote in USD for Codex10k tracking but buyer budget is CAD.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Canadian nonprofit; quote in USD for Codex10k tracking but buyer budget is CAD.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">

</xml_diff>

<commit_message>
Prepare Codex10k prep draft packets
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R8d64cef1e09a4cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R1ee43fbe66274aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R6200f806ceec486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rb3404269fa9f42a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5f5a66bafe3c44f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0c307bdf51e74b8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R77228d5a01f247b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra37b497c29b84d78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>99</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5549,6 +5549,346 @@
         <x:v>Follow-up draft only. Do not send immediately unless user wants a manual follow-up cadence.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>C10K-104</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Claire Manwaring / caregiver SMS workflow</x:v>
+      </x:c>
+      <x:c r="E105"/>
+      <x:c r="F105" t="str">
+        <x:v>Make Community draft</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>https://community.make.com/t/looking-for-short-term-help-with-make-bubble-supabase-claude-twilio/108581</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>Caregiver SMS workflow</x:v>
+      </x:c>
+      <x:c r="I105" t="str">
+        <x:v>The risk is not one Make scenario; it is durable conversation state, approval routing, audit logs, analytics, and safe escalation boundaries.</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>Stateful SMS MVP build-readiness sprint</x:v>
+      </x:c>
+      <x:c r="K105" t="str">
+        <x:v>prep_draft_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L105" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M105" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to Claire_Manwaring</x:v>
+      </x:c>
+      <x:c r="N105" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O105" t="str">
+        <x:v>c10k-104-claire-manwaring-caregiver-sms-workflow.html; outputs/codex10k/prep-drafts/c10k-104-claire-manwaring-caregiver-sms-workflow.pdf; outputs/codex10k/prep-drafts/c10k-104-claire-manwaring-caregiver-sms-workflow.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-104-claire-manwaring-caregiver-sms-workflow.html?v=prep2</x:v>
+      </x:c>
+      <x:c r="P105" t="str">
+        <x:v>Forum/DM path only unless Claire provides an email. Do not request PHI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>C10K-105</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Ray Roberts / HubSpot document export</x:v>
+      </x:c>
+      <x:c r="E106"/>
+      <x:c r="F106" t="str">
+        <x:v>Make Community draft</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>https://community.make.com/t/looking-for-help-with-export-documents-from-hubspot-to-nutshell-or-just-export/108371</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>CRM document migration</x:v>
+      </x:c>
+      <x:c r="I106" t="str">
+        <x:v>The buyer needs an inventory, sample transfer/export, manifest, and failure report before committing to a full migration run.</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>HubSpot document rescue sprint</x:v>
+      </x:c>
+      <x:c r="K106" t="str">
+        <x:v>prep_draft_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L106" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M106" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to RayRoberts</x:v>
+      </x:c>
+      <x:c r="N106" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O106" t="str">
+        <x:v>c10k-105-ray-roberts-hubspot-document-export.html; outputs/codex10k/prep-drafts/c10k-105-ray-roberts-hubspot-document-export.pdf; outputs/codex10k/prep-drafts/c10k-105-ray-roberts-hubspot-document-export.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-105-ray-roberts-hubspot-document-export.html?v=prep2</x:v>
+      </x:c>
+      <x:c r="P106" t="str">
+        <x:v>Forum/DM path only unless Ray provides an email. Verify Nutshell attachment support before promising transfer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>C10K-106</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>Eli Malone-Shkurkin / research automation</x:v>
+      </x:c>
+      <x:c r="E107"/>
+      <x:c r="F107" t="str">
+        <x:v>Make Community draft</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>https://community.make.com/t/looking-to-hire-pro-for-daily-industry-research-automation-40-hours-good-rates/107995</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>AI research workflow</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>The current workflow likely benefits from a client config layer, persistence cleanup, failure logging, and output provisioning before it scales.</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>Self-serve research automation upgrade</x:v>
+      </x:c>
+      <x:c r="K107" t="str">
+        <x:v>prep_draft_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L107" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to Eli_Malone-Shkurkin</x:v>
+      </x:c>
+      <x:c r="N107" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O107" t="str">
+        <x:v>c10k-106-eli-malone-shkurkin-research-automation.html; outputs/codex10k/prep-drafts/c10k-106-eli-malone-shkurkin-research-automation.pdf; outputs/codex10k/prep-drafts/c10k-106-eli-malone-shkurkin-research-automation.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-106-eli-malone-shkurkin-research-automation.html?v=prep2</x:v>
+      </x:c>
+      <x:c r="P107" t="str">
+        <x:v>Forum/DM path only unless Eli provides an email. Keep data-source permissions explicit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>C10K-107</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>birthcoachuk / Marley</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>marley@midwifemarley.com</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Bubble Forum / public email draft</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>https://forum.bubble.io/t/experienced-bubble-developer-needed-for-saas-mvp/393713</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>Bubble SaaS architecture</x:v>
+      </x:c>
+      <x:c r="I108" t="str">
+        <x:v>The full build is compliance-sensitive; the safest first close is a technical blueprint and milestone quote before implementation.</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>Bubble SaaS technical blueprint + build plan</x:v>
+      </x:c>
+      <x:c r="K108" t="str">
+        <x:v>gmail_draft_created_no_send</x:v>
+      </x:c>
+      <x:c r="L108" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M108" t="str">
+        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+      </x:c>
+      <x:c r="N108" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O108" t="str">
+        <x:v>c10k-107-birthcoachuk-marley.html; outputs/codex10k/prep-drafts/c10k-107-birthcoachuk-marley.pdf; outputs/codex10k/prep-drafts/c10k-107-birthcoachuk-marley.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-107-birthcoachuk-marley.html?v=prep2; gmail_draft:r5078376235347498872; gmail_msg:19e11896d51706b1</x:v>
+      </x:c>
+      <x:c r="P108" t="str">
+        <x:v>Created Gmail draft only; no send. Public email listed in Bubble Forum post; discovery/blueprint scope only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>C10K-108</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Town of Parker / PACE</x:v>
+      </x:c>
+      <x:c r="E109"/>
+      <x:c r="F109" t="str">
+        <x:v>Bonfire portal packet</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>https://parkeronline.bonfirehub.com/opportunities/232506</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>Scheduling system data migration</x:v>
+      </x:c>
+      <x:c r="I109" t="str">
+        <x:v>Scheduling replacement risk is concentrated around legacy data inventory, field mapping, duplicate rules, migration tests, and cutover evidence.</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>Legacy scheduling data migration readiness pack</x:v>
+      </x:c>
+      <x:c r="K109" t="str">
+        <x:v>prep_draft_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L109" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M109" t="str">
+        <x:v>Review prepared packet and use only via approved path: Bonfire/Euna portal only</x:v>
+      </x:c>
+      <x:c r="N109" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O109" t="str">
+        <x:v>c10k-108-town-of-parker-pace.html; outputs/codex10k/prep-drafts/c10k-108-town-of-parker-pace.pdf; outputs/codex10k/prep-drafts/c10k-108-town-of-parker-pace.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-108-town-of-parker-pace.html?v=prep2</x:v>
+      </x:c>
+      <x:c r="P109" t="str">
+        <x:v>Portal-only. Do not send casual email or submit without action-time approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>C10K-109</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>City of Raleigh Planning &amp; Development</x:v>
+      </x:c>
+      <x:c r="E110"/>
+      <x:c r="F110" t="str">
+        <x:v>NC eVP portal packet</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>https://evp.nc.gov/solicitations/</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>M365 / records governance</x:v>
+      </x:c>
+      <x:c r="I110" t="str">
+        <x:v>The practical first win is a pilot inventory/taxonomy/permissions workflow that proves governance before citywide rollout.</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>M365 and SharePoint information governance pilot</x:v>
+      </x:c>
+      <x:c r="K110" t="str">
+        <x:v>prep_draft_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L110" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M110" t="str">
+        <x:v>Review prepared packet and use only via approved path: NC electronic Vendor Portal</x:v>
+      </x:c>
+      <x:c r="N110" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O110" t="str">
+        <x:v>c10k-109-city-of-raleigh-planning-development.html; outputs/codex10k/prep-drafts/c10k-109-city-of-raleigh-planning-development.pdf; outputs/codex10k/prep-drafts/c10k-109-city-of-raleigh-planning-development.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-109-city-of-raleigh-planning-development.html?v=prep2</x:v>
+      </x:c>
+      <x:c r="P110" t="str">
+        <x:v>Portal-only. Do not send or submit without action-time approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>C10K-110</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>MORPC - Central Ohio Transportation Safety and Non-Motorized Data Collection Plans</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>mschaper@morpc.org</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>MPO RFP email draft</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>https://www.morpc.org/wp-content/uploads/2026/04/RFP-Central-Ohio-Transportation-Safety-Plan.pdf</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>Transportation safety data</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>A narrow dashboard/data workflow support slice can help the prime team turn counts, crash data, and VRU priorities into repeatable update evidence.</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>Safety dashboard prototype + update workflow support</x:v>
+      </x:c>
+      <x:c r="K111" t="str">
+        <x:v>gmail_draft_created_no_send</x:v>
+      </x:c>
+      <x:c r="L111" t="str">
+        <x:v>2026-05-10</x:v>
+      </x:c>
+      <x:c r="M111" t="str">
+        <x:v>User review in Gmail drafts; send manually only if desired after formal path review. No automated send occurred.</x:v>
+      </x:c>
+      <x:c r="N111" t="str">
+        <x:v>2026-05-13</x:v>
+      </x:c>
+      <x:c r="O111" t="str">
+        <x:v>c10k-110-morpc-central-ohio-transportation-safety-and-non-motorized-data-collection-plans.html; outputs/codex10k/prep-drafts/c10k-110-morpc-central-ohio-transportation-safety-and-non-motorized-data-collection-plans.pdf; outputs/codex10k/prep-drafts/c10k-110-morpc-central-ohio-transportation-safety-and-non-motorized-data-collection-plans.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-110-morpc-central-ohio-transportation-safety-and-non-motorized-data-collection-plans.html?v=prep2; gmail_draft:r8406472525554024594; gmail_msg:19e1189af82c22e8</x:v>
+      </x:c>
+      <x:c r="P111" t="str">
+        <x:v>Created Gmail draft only; no send. Use only as prime/subconsultant collateral or formal compliant proposal path after approval.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Send ABMC Codex10k draft
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R5f5a66bafe3c44f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R0c307bdf51e74b8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R77228d5a01f247b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra37b497c29b84d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R311eecbac1764a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Reca082b3bcc645ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R00eb75418d7340c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbf02e6d630744b26"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4731,22 +4731,22 @@
         <x:v>HRIS migration and acceptance QA support</x:v>
       </x:c>
       <x:c r="K88" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L88" t="str">
-        <x:v>2026-05-10</x:v>
+        <x:v>2026-05-11</x:v>
       </x:c>
       <x:c r="M88" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for reply; if positive, route through ABMC federal or prime/subcontract procurement path before any invoice/payment link.</x:v>
       </x:c>
       <x:c r="N88" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-14</x:v>
       </x:c>
       <x:c r="O88" t="str">
-        <x:v>c10k-087-american-battle-monuments-commission.html; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.pdf; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-087-american-battle-monuments-commission.html?v=draft1; gmail_draft:r8757273967754748544; gmail_msg:19e1132cd3f3895f</x:v>
+        <x:v>c10k-087-american-battle-monuments-commission.html; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.pdf; outputs/codex10k/draft-batch/c10k-087-american-battle-monuments-commission.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-087-american-battle-monuments-commission.html?v=draft1; gmail_draft:r8757273967754748544; gmail_msg:19e1132cd3f3895f; gmail_sent:19e14b5fa14e435a</x:v>
       </x:c>
       <x:c r="P88" t="str">
-        <x:v>Federal HRIS. Avoid PII and avoid implying this is the full HRIS proposal.</x:v>
+        <x:v>Federal HRIS. Avoid PII and avoid implying this is the full HRIS proposal. Sent from prepared draft on 2026-05-11T01:45:39Z; thread:19e1132cd3f3895f; support slice only, no employee PII, no full HRIS prime claim.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4831,22 +4831,22 @@
         <x:v>GIS/data workflow QA and deliverable support slice</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>sent_from_draft</x:v>
+        <x:v>auto_reply_received</x:v>
       </x:c>
       <x:c r="L90" t="str">
         <x:v>2026-05-10</x:v>
       </x:c>
       <x:c r="M90" t="str">
-        <x:v>Watch for reply; if positive, use docs/draft-payment-close-pack.md and confirm support/teaming path before any payment link/invoice</x:v>
+        <x:v>No action from auto-reply; wait for human response or consider one polite follow-up after May 13 if still relevant.</x:v>
       </x:c>
       <x:c r="N90" t="str">
         <x:v>2026-05-13</x:v>
       </x:c>
       <x:c r="O90" t="str">
-        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1; gmail_draft:r-3371871953269203560; gmail_msg:19e11337718ef02e; gmail_sent:19e116d0b7e2a01a</x:v>
+        <x:v>c10k-089-town-of-hillsborough.html; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.pdf; outputs/codex10k/draft-batch/c10k-089-town-of-hillsborough.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-089-town-of-hillsborough.html?v=draft1; gmail_draft:r-3371871953269203560; gmail_msg:19e11337718ef02e; gmail_sent:19e116d0b7e2a01a; gmail_auto_reply:19e116d7c935aee2</x:v>
       </x:c>
       <x:c r="P90" t="str">
-        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Do not imply engineering credentials; support/teaming path only.</x:v>
+        <x:v>Sent from Gmail draft after one-time user approval to bypass 15-minute guard for the 7-mail batch. Do not imply engineering credentials; support/teaming path only. Received out-of-office auto-reply from Doug Belcik on 2026-05-10T10:27:26Z saying he was away until Monday May 11; not a buying signal.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">

</xml_diff>

<commit_message>
Prepare May 11 Codex10k packet batch
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R311eecbac1764a7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Reca082b3bcc645ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R00eb75418d7340c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Rbf02e6d630744b26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc2a27036765147a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4fda2dd788eb4b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rcb0e7ec1d7e54cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra22019eaf2d643cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIFS(Prospects!K2:K200,"&lt;&gt;initialized",Prospects!K2:K200,"&lt;&gt;hold_employment_style",Prospects!K2:K200,"&lt;&gt;bounced",Prospects!K2:K200,"&lt;&gt;")</x:f>
-        <x:v>106</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -5889,6 +5889,534 @@
         <x:v>Created Gmail draft only; no send. Use only as prime/subconsultant collateral or formal compliant proposal path after approval.</x:v>
       </x:c>
     </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>C10K-111</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>City of Boston - Identity and Access Management Managed Services</x:v>
+      </x:c>
+      <x:c r="E112"/>
+      <x:c r="F112" t="str">
+        <x:v>Boston Supplier Portal packet</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>https://content.boston.gov/bid-listings/ev00017196</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>IAM UAT and proposal readiness</x:v>
+      </x:c>
+      <x:c r="I112" t="str">
+        <x:v>A prime bidder can use a compact UAT/control-evidence appendix to strengthen implementation readiness without overclaiming prime IAM capacity.</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>IAM proposal readiness and UAT evidence pack</x:v>
+      </x:c>
+      <x:c r="K112" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L112" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M112" t="str">
+        <x:v>Review prepared packet and use only via approved path: Boston Supplier Portal or approved prime/subcontract path</x:v>
+      </x:c>
+      <x:c r="N112" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O112" t="str">
+        <x:v>c10k-111-city-of-boston-identity-and-access-management-managed-services.html; outputs/codex10k/may11-prep-batch/c10k-111-city-of-boston-identity-and-access-management-managed-services.pdf; outputs/codex10k/may11-prep-batch/c10k-111-city-of-boston-identity-and-access-management-managed-services.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-111-city-of-boston-identity-and-access-management-managed-services.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P112" t="str">
+        <x:v>Portal-only for buyer submission. Gmail only for procedural clarification to the named contact, not sales outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>C10K-112</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>City of St. Cloud - ERP Software and Implementation Services</x:v>
+      </x:c>
+      <x:c r="E113"/>
+      <x:c r="F113" t="str">
+        <x:v>OpenGov portal packet</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>https://govtribe.com/opportunity/state-local-contract-opportunity/enterprise-resource-planning-erp-software-and-implementation-services-2026027</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>ERP data migration and UAT</x:v>
+      </x:c>
+      <x:c r="I113" t="str">
+        <x:v>ERP implementation risk is concentrated in conversion inventory, interface assumptions, UAT coverage, and cutover evidence.</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>ERP data conversion and UAT readiness sidecar</x:v>
+      </x:c>
+      <x:c r="K113" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L113" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M113" t="str">
+        <x:v>Review prepared packet and use only via approved path: St. Cloud OpenGov portal or approved ERP prime/subcontract path</x:v>
+      </x:c>
+      <x:c r="N113" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O113" t="str">
+        <x:v>c10k-112-city-of-st-cloud-erp-software-and-implementation-services.html; outputs/codex10k/may11-prep-batch/c10k-112-city-of-st-cloud-erp-software-and-implementation-services.pdf; outputs/codex10k/may11-prep-batch/c10k-112-city-of-st-cloud-erp-software-and-implementation-services.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-112-city-of-st-cloud-erp-software-and-implementation-services.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P113" t="str">
+        <x:v>Portal-only to the agency. Gmail is appropriate only for approved ERP vendor/prime teaming outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>C10K-113</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>City of San Antonio Public Library - Digital Experience Redesign</x:v>
+      </x:c>
+      <x:c r="E114"/>
+      <x:c r="F114" t="str">
+        <x:v>SAePS portal packet</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>https://webapp1.sanantonio.gov/BidContractOpps/Content.aspx?id=6163&amp;page=Default</x:v>
+      </x:c>
+      <x:c r="H114" t="str">
+        <x:v>Digital library launch QA</x:v>
+      </x:c>
+      <x:c r="I114" t="str">
+        <x:v>The most useful support slice is acceptance evidence across patron journeys, accessibility, search, account flows, and admin workflows.</x:v>
+      </x:c>
+      <x:c r="J114" t="str">
+        <x:v>Digital library accessibility and launch acceptance test pack</x:v>
+      </x:c>
+      <x:c r="K114" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L114" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M114" t="str">
+        <x:v>Review prepared packet and use only via approved path: SAePS portal or approved selected-vendor/prime path</x:v>
+      </x:c>
+      <x:c r="N114" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O114" t="str">
+        <x:v>c10k-113-city-of-san-antonio-public-library-digital-experience-redesign.html; outputs/codex10k/may11-prep-batch/c10k-113-city-of-san-antonio-public-library-digital-experience-redesign.pdf; outputs/codex10k/may11-prep-batch/c10k-113-city-of-san-antonio-public-library-digital-experience-redesign.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-113-city-of-san-antonio-public-library-digital-experience-redesign.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P114" t="str">
+        <x:v>Portal-only. Do not Gmail or cold-email outside listed solicitation communication rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>C10K-114</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>WSSC Water - GIS and Engineering Records Document Management Support</x:v>
+      </x:c>
+      <x:c r="E115"/>
+      <x:c r="F115" t="str">
+        <x:v>OpenGov portal packet</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>https://procurement.opengov.com/portal/wsscwater/projects/256299</x:v>
+      </x:c>
+      <x:c r="H115" t="str">
+        <x:v>GIS, ECM, and engineering records</x:v>
+      </x:c>
+      <x:c r="I115" t="str">
+        <x:v>The first value is a task-order starter pack that maps likely use cases, data/workflow risks, and staffing evidence for a BOA response.</x:v>
+      </x:c>
+      <x:c r="J115" t="str">
+        <x:v>GIS/ECM readiness and task-order starter pack</x:v>
+      </x:c>
+      <x:c r="K115" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L115" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M115" t="str">
+        <x:v>Review prepared packet and use only via approved path: WSSC OpenGov portal or approved prime/subcontract path</x:v>
+      </x:c>
+      <x:c r="N115" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O115" t="str">
+        <x:v>c10k-114-wssc-water-gis-and-engineering-records-document-management-support.html; outputs/codex10k/may11-prep-batch/c10k-114-wssc-water-gis-and-engineering-records-document-management-support.pdf; outputs/codex10k/may11-prep-batch/c10k-114-wssc-water-gis-and-engineering-records-document-management-support.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-114-wssc-water-gis-and-engineering-records-document-management-support.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P115" t="str">
+        <x:v>Portal-only for buyer. Gmail only for approved teaming outreach to likely primes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>C10K-115</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>City of St. Petersburg - Pension Management Software</x:v>
+      </x:c>
+      <x:c r="E116"/>
+      <x:c r="F116" t="str">
+        <x:v>OpenGov portal packet</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>https://procurement.opengov.com/portal/stpete</x:v>
+      </x:c>
+      <x:c r="H116" t="str">
+        <x:v>Pension SaaS fit-gap and workflow QA</x:v>
+      </x:c>
+      <x:c r="I116" t="str">
+        <x:v>A fit-gap and demo-script pack can help evaluate vendor responses and surface migration/reporting risk before award.</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>Pension data and workflow fit-gap sprint</x:v>
+      </x:c>
+      <x:c r="K116" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L116" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M116" t="str">
+        <x:v>Review prepared packet and use only via approved path: St. Petersburg OpenGov portal or approved vendor/prime path</x:v>
+      </x:c>
+      <x:c r="N116" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O116" t="str">
+        <x:v>c10k-115-city-of-st-petersburg-pension-management-software.html; outputs/codex10k/may11-prep-batch/c10k-115-city-of-st-petersburg-pension-management-software.pdf; outputs/codex10k/may11-prep-batch/c10k-115-city-of-st-petersburg-pension-management-software.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-115-city-of-st-petersburg-pension-management-software.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P116" t="str">
+        <x:v>Portal-only to the agency. Procedural email only if permitted by the solicitation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>C10K-116</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>South Carolina Governor's School for Science and Mathematics</x:v>
+      </x:c>
+      <x:c r="E117"/>
+      <x:c r="F117" t="str">
+        <x:v>South Carolina procurement packet</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>https://apps.sceis.sc.gov/SCSolicitationWeb/solicitationAttachment.do?solicitnumber=5400028226</x:v>
+      </x:c>
+      <x:c r="H117" t="str">
+        <x:v>School website CMS and security response</x:v>
+      </x:c>
+      <x:c r="I117" t="str">
+        <x:v>The support lane is a response pack around CMS support, security evidence mapping, WCAG plan, integration inventory, and redacted-copy QA.</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>CMS support and accessibility/security response pack</x:v>
+      </x:c>
+      <x:c r="K117" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L117" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M117" t="str">
+        <x:v>Review prepared packet and use only via approved path: South Carolina procurement portal or approved web/CMS prime path</x:v>
+      </x:c>
+      <x:c r="N117" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O117" t="str">
+        <x:v>c10k-116-south-carolina-governor-s-school-for-science-and-mathematics.html; outputs/codex10k/may11-prep-batch/c10k-116-south-carolina-governor-s-school-for-science-and-mathematics.pdf; outputs/codex10k/may11-prep-batch/c10k-116-south-carolina-governor-s-school-for-science-and-mathematics.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-116-south-carolina-governor-s-school-for-science-and-mathematics.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P117" t="str">
+        <x:v>Portal-only. Email only for formal procurement questions, not sales outreach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>C10K-117</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Northside Independent School District - District Web Services</x:v>
+      </x:c>
+      <x:c r="E118"/>
+      <x:c r="F118" t="str">
+        <x:v>Bonfire/Euna portal packet</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>https://media.governmentnavigator.com/media/bid/1776452898_4_17_2026-2026-070.pdf</x:v>
+      </x:c>
+      <x:c r="H118" t="str">
+        <x:v>District web compliance support</x:v>
+      </x:c>
+      <x:c r="I118" t="str">
+        <x:v>A tight compliance sidecar can help a web prime complete the SOW questionnaire, accessibility/security matrix, FERPA/data-transfer checklist, and portal package QA.</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>District web RFP compliance sidecar</x:v>
+      </x:c>
+      <x:c r="K118" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L118" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M118" t="str">
+        <x:v>Review prepared packet and use only via approved path: NISD Bonfire/Euna portal or approved district web prime path</x:v>
+      </x:c>
+      <x:c r="N118" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O118" t="str">
+        <x:v>c10k-117-northside-independent-school-district-district-web-services.html; outputs/codex10k/may11-prep-batch/c10k-117-northside-independent-school-district-district-web-services.pdf; outputs/codex10k/may11-prep-batch/c10k-117-northside-independent-school-district-district-web-services.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-117-northside-independent-school-district-district-web-services.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P118" t="str">
+        <x:v>Portal-only. No Gmail outreach during procurement evaluation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>C10K-118</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>NJ TRANSIT - Rail Origin-Destination Survey</x:v>
+      </x:c>
+      <x:c r="E119"/>
+      <x:c r="F119" t="str">
+        <x:v>Bid Express support packet</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>https://www.njtransit.com/procurement/calendar/</x:v>
+      </x:c>
+      <x:c r="H119" t="str">
+        <x:v>Transportation survey data QA</x:v>
+      </x:c>
+      <x:c r="I119" t="str">
+        <x:v>A subconsultant support slice can cover schema QA, cleaning rules, dashboard wireframes, and field-to-analysis handoff evidence.</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>O-D survey data QA and dashboard prototype</x:v>
+      </x:c>
+      <x:c r="K119" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L119" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M119" t="str">
+        <x:v>Review prepared packet and use only via approved path: Bid Express or approved survey/planning prime path</x:v>
+      </x:c>
+      <x:c r="N119" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O119" t="str">
+        <x:v>c10k-118-nj-transit-rail-origin-destination-survey.html; outputs/codex10k/may11-prep-batch/c10k-118-nj-transit-rail-origin-destination-survey.pdf; outputs/codex10k/may11-prep-batch/c10k-118-nj-transit-rail-origin-destination-survey.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-118-nj-transit-rail-origin-destination-survey.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P119" t="str">
+        <x:v>Portal-only to NJ TRANSIT. Gmail only for approved teaming outreach to survey/planning primes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>C10K-119</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Brittany / nonprofit Salesforce-ActiveCampaign Make scenarios</x:v>
+      </x:c>
+      <x:c r="E120"/>
+      <x:c r="F120" t="str">
+        <x:v>Make Community forum packet</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>https://community.make.com/t/need-help-with-integrations-on-scenarios/107903</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>CRM integration rescue</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>The practical first close is stabilizing two scenarios with mapping rules, dedupe checks, error handling, and a short runbook.</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>Salesforce-ActiveCampaign Make stabilization sprint</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to Brittany</x:v>
+      </x:c>
+      <x:c r="N120" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O120" t="str">
+        <x:v>c10k-119-brittany-nonprofit-salesforce-activecampaign-make-scenarios.html; outputs/codex10k/may11-prep-batch/c10k-119-brittany-nonprofit-salesforce-activecampaign-make-scenarios.pdf; outputs/codex10k/may11-prep-batch/c10k-119-brittany-nonprofit-salesforce-activecampaign-make-scenarios.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-119-brittany-nonprofit-salesforce-activecampaign-make-scenarios.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P120" t="str">
+        <x:v>Forum/DM only unless Brittany provides a public email. Do not request donor/member data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>C10K-120</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Emanuel Arias - Notion and Adalo integration</x:v>
+      </x:c>
+      <x:c r="E121"/>
+      <x:c r="F121" t="str">
+        <x:v>Make Community forum packet</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>https://community.make.com/t/help-setting-up-a-notion-adalo-app-integration/107803</x:v>
+      </x:c>
+      <x:c r="H121" t="str">
+        <x:v>No-code app data sync</x:v>
+      </x:c>
+      <x:c r="I121" t="str">
+        <x:v>A one-direction sync with upsert, dedupe, and error logging is the safest first version before promising two-way behavior.</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>Notion-Adalo Sync v1</x:v>
+      </x:c>
+      <x:c r="K121" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L121" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M121" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to Emanuel_Arias</x:v>
+      </x:c>
+      <x:c r="N121" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O121" t="str">
+        <x:v>c10k-120-emanuel-arias-notion-and-adalo-integration.html; outputs/codex10k/may11-prep-batch/c10k-120-emanuel-arias-notion-and-adalo-integration.pdf; outputs/codex10k/may11-prep-batch/c10k-120-emanuel-arias-notion-and-adalo-integration.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-120-emanuel-arias-notion-and-adalo-integration.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P121" t="str">
+        <x:v>Forum/DM only. Do not request live API tokens in messages.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>C10K-121</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>Codex10k</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Ann - Make, Typebot, OpenAI, and Airtable setup</x:v>
+      </x:c>
+      <x:c r="E122"/>
+      <x:c r="F122" t="str">
+        <x:v>Make Community forum packet</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>https://community.make.com/t/integration-make-typebot-open-ai-airtable/107562</x:v>
+      </x:c>
+      <x:c r="H122" t="str">
+        <x:v>AI chatbot workflow rescue</x:v>
+      </x:c>
+      <x:c r="I122" t="str">
+        <x:v>The fastest useful paid task is fixing permissions/model access and proving one working multi-step bot flow with Airtable read/write.</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>Typebot-Airtable-AI setup rescue</x:v>
+      </x:c>
+      <x:c r="K122" t="str">
+        <x:v>prep_packet_ready_no_send</x:v>
+      </x:c>
+      <x:c r="L122" t="str">
+        <x:v>2026-05-11</x:v>
+      </x:c>
+      <x:c r="M122" t="str">
+        <x:v>Review prepared packet and use only via approved path: Make Community reply/DM to Ann</x:v>
+      </x:c>
+      <x:c r="N122" t="str">
+        <x:v>2026-05-14</x:v>
+      </x:c>
+      <x:c r="O122" t="str">
+        <x:v>c10k-121-ann-make-typebot-openai-and-airtable-setup.html; outputs/codex10k/may11-prep-batch/c10k-121-ann-make-typebot-openai-and-airtable-setup.pdf; outputs/codex10k/may11-prep-batch/c10k-121-ann-make-typebot-openai-and-airtable-setup.draft.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-121-ann-make-typebot-openai-and-airtable-setup.html?v=may11prep</x:v>
+      </x:c>
+      <x:c r="P122" t="str">
+        <x:v>Forum/DM only. Never request API keys over forum or email.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Send BakerRipley eligibility question
</commit_message>
<xml_diff>
--- a/outputs/codex10k/codex10k_revenue_tracker.xlsx
+++ b/outputs/codex10k/codex10k_revenue_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc2a27036765147a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="R4fda2dd788eb4b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="Rcb0e7ec1d7e54cf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra22019eaf2d643cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6170f34de9f74613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ledger" sheetId="2" r:id="Rb5bee894b5d44abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" r:id="R9eadafe313ac444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="Ra417b5990585493b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4581,22 +4581,22 @@
         <x:v>Salesforce implementation QA and UAT support sidecar</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>gmail_draft_created_no_send</x:v>
+        <x:v>sent_from_draft</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>2026-05-10</x:v>
+        <x:v>2026-05-11</x:v>
       </x:c>
       <x:c r="M85" t="str">
-        <x:v>User review in Gmail drafts; send manually only if desired. No automated send occurred.</x:v>
+        <x:v>Watch for BakerRipley eligibility reply; if positive, confirm procurement/support-sidecar path before any invoice or payment link.</x:v>
       </x:c>
       <x:c r="N85" t="str">
-        <x:v>2026-05-13</x:v>
+        <x:v>2026-05-14</x:v>
       </x:c>
       <x:c r="O85" t="str">
-        <x:v>c10k-084-bakerripley.html; outputs/codex10k/draft-batch/c10k-084-bakerripley.pdf; outputs/codex10k/draft-batch/c10k-084-bakerripley.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-084-bakerripley.html?v=draft1; gmail_draft:r7718642615731016285; gmail_msg:19e1131cdbe3bdaf</x:v>
+        <x:v>c10k-084-bakerripley.html; outputs/codex10k/draft-batch/c10k-084-bakerripley.pdf; outputs/codex10k/draft-batch/c10k-084-bakerripley.email.txt; https://anonymusk7.github.io/codex10k-workflow-recovery/c10k-084-bakerripley.html?v=draft1; gmail_draft:r7718642615731016285; gmail_msg:19e1131cdbe3bdaf; gmail_sent:19e14dcf92e67eb9</x:v>
       </x:c>
       <x:c r="P85" t="str">
-        <x:v>Mandatory vendor conference risk. This draft asks eligibility before proposing work.</x:v>
+        <x:v>Mandatory vendor conference risk. This draft asks eligibility before proposing work. Sent from prepared draft on 2026-05-11T02:28:16Z; thread:19e1131cdbe3bdaf; eligibility question only because May 5 vendor conference may have been mandatory.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">

</xml_diff>